<commit_message>
feat: URLs statiques PDF pour les 33 lots, integration automatique dans les messages WhatsApp et redirection 1-clic wa.me dans le fichier Excel
</commit_message>
<xml_diff>
--- a/data/Résidence BELLES LOGES-2026.xlsx
+++ b/data/Résidence BELLES LOGES-2026.xlsx
@@ -28,7 +28,7 @@
     <numFmt numFmtId="166" formatCode="#,##0\ &quot;DH&quot;;[Red]\-#,##0\ &quot;DH&quot;"/>
     <numFmt numFmtId="167" formatCode="_-* #,##0.00\ _€_-;\-* #,##0.00\ _€_-;_-* &quot;-&quot;??\ _€_-;_-@_-"/>
   </numFmts>
-  <fonts count="33">
+  <fonts count="36">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -263,8 +263,28 @@
       <b val="1"/>
       <sz val="14"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000284C7"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="0016A34A"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
   </fonts>
-  <fills count="20">
+  <fills count="22">
     <fill>
       <patternFill/>
     </fill>
@@ -378,6 +398,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E293B"/>
+        <bgColor rgb="001E293B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00166534"/>
+        <bgColor rgb="00166534"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="68">
     <border>
@@ -1246,7 +1278,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="265">
+  <cellXfs count="269">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1996,6 +2028,14 @@
     <xf numFmtId="164" fontId="23" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
+    <xf numFmtId="0" fontId="33" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2869,6 +2909,10 @@
     <col width="21.42578125" customWidth="1" min="20" max="20"/>
     <col width="24.85546875" bestFit="1" customWidth="1" min="21" max="21"/>
     <col width="27" customWidth="1" min="22" max="22"/>
+    <col width="20" customWidth="1" min="23" max="23"/>
+    <col width="30" customWidth="1" min="24" max="24"/>
+    <col width="45" customWidth="1" min="25" max="25"/>
+    <col width="25" customWidth="1" min="26" max="26"/>
     <col width="9.5703125" bestFit="1" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
@@ -2990,6 +3034,26 @@
           <t>Les arriérés 2024</t>
         </is>
       </c>
+      <c r="W6" s="265" t="inlineStr">
+        <is>
+          <t>Lien PDF Statique</t>
+        </is>
+      </c>
+      <c r="X6" s="266" t="inlineStr">
+        <is>
+          <t>📲 ENVOYER WHATSAPP (1-CLIC)</t>
+        </is>
+      </c>
+      <c r="Y6" s="265" t="inlineStr">
+        <is>
+          <t>Message WhatsApp Prêt</t>
+        </is>
+      </c>
+      <c r="Z6" s="265" t="inlineStr">
+        <is>
+          <t>Lien Espace Client Direct</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="24.95" customHeight="1">
       <c r="B7" s="122" t="inlineStr">
@@ -3064,6 +3128,37 @@
         <f>'Cotisation 2025'!V7</f>
         <v/>
       </c>
+      <c r="W7" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/pdf/appel-M01.pdf", "📄 Voir PDF (M01)")</f>
+        <v/>
+      </c>
+      <c r="X7" s="268">
+        <f>HYPERLINK("https://wa.me/212669281802?text=%F0%9F%8F%A2%20%2ASYNDICAT%20R%C3%89SIDENCE%20BELLES%20LOGES%2A%0A%F0%9F%93%8D%20Rue%20Attabari%2C%20Quartier%20Les%20Princesses%2C%20Casablanca%0A%0ABonjour%20%2ANMJ%20CAPITAL%2A%2C%0A%0AVeuillez%20trouver%20ci-dessous%20l%27appel%20de%20cotisations%20syndicales%20pour%20votre%20bien%20%28%2AMagasin%20N%C2%B0%201%2A%20/%20M01%29%20%3A%0A%0A%F0%9F%93%85%20%2AP%C3%A9riode%20%3A%2A%20Ann%C3%A9e%202026%0A%F0%9F%92%B0%20%2ATotal%20%C3%A0%20r%C3%A9gler%20%3A%2A%20%2A1800%20DH%2A%0A%0A%F0%9F%93%84%20%2AT%C3%A9l%C3%A9charger%20votre%20document%20officiel%20%28PDF%29%20%3A%2A%0A%F0%9F%91%89%20https%3A//srbl.netlify.app/pdf/appel-M01.pdf%0A%0A%F0%9F%8F%A6%20%2ACoordonn%C3%A9es%20bancaires%20pour%20le%20virement%20%3A%2A%0A%E2%80%A2%20%2AB%C3%A9n%C3%A9ficiaire%20%3A%2A%20SYNDICAT%20RESIDENCE%20BELLES%20LOGES%0A%E2%80%A2%20%2ABanque%20%3A%2A%20BMCE%20/%20BANK%20OF%20AFRICA%0A%E2%80%A2%20%2ARIB%20%3A%2A%20%60011%20780%200000402100011545%2025%60%0A%0A_Motif%20%3A%20M01%20-%20NMJ%20CAPITAL_%0A%0AMerci%20pour%20votre%20pr%C3%A9cieuse%20collaboration.%0A%2ALe%20Bureau%20du%20Syndic%2A", "📲 Envoyer WhatsApp Direct")</f>
+        <v/>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>🏢 *SYNDICAT RÉSIDENCE BELLES LOGES*
+📍 Rue Attabari, Quartier Les Princesses, Casablanca
+Bonjour *NMJ CAPITAL*,
+Veuillez trouver ci-dessous l'appel de cotisations syndicales pour votre bien (*Magasin N° 1* / M01) :
+📅 *Période :* Année 2026
+💰 *Total à régler :* *1800 DH*
+📄 *Télécharger votre document officiel (PDF) :*
+👉 https://srbl.netlify.app/pdf/appel-M01.pdf
+🏦 *Coordonnées bancaires pour le virement :*
+• *Bénéficiaire :* SYNDICAT RESIDENCE BELLES LOGES
+• *Banque :* BMCE / BANK OF AFRICA
+• *RIB :* `011 780 0000402100011545 25`
+_Motif : M01 - NMJ CAPITAL_
+Merci pour votre précieuse collaboration.
+*Le Bureau du Syndic*</t>
+        </is>
+      </c>
+      <c r="Z7" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/?client=M01", "👤 Espace Client (M01)")</f>
+        <v/>
+      </c>
     </row>
     <row r="8" ht="24.95" customHeight="1">
       <c r="B8" s="128" t="inlineStr">
@@ -3137,6 +3232,37 @@
         <f>'Cotisation 2025'!V8</f>
         <v/>
       </c>
+      <c r="W8" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/pdf/appel-M02.pdf", "📄 Voir PDF (M02)")</f>
+        <v/>
+      </c>
+      <c r="X8" s="268">
+        <f>HYPERLINK("https://wa.me/212669791313?text=%F0%9F%8F%A2%20%2ASYNDICAT%20R%C3%89SIDENCE%20BELLES%20LOGES%2A%0A%F0%9F%93%8D%20Rue%20Attabari%2C%20Quartier%20Les%20Princesses%2C%20Casablanca%0A%0ABonjour%20%2AHIND%20DRIOUECH%20ET%20MR%20ABDELAH%20NACHIT%2A%2C%0A%0AVeuillez%20trouver%20ci-dessous%20l%27appel%20de%20cotisations%20syndicales%20pour%20votre%20bien%20%28%2AMagasin%20N%C2%B0%202%2A%20/%20M02%29%20%3A%0A%0A%F0%9F%93%85%20%2AP%C3%A9riode%20%3A%2A%20Ann%C3%A9e%202026%0A%F0%9F%92%B0%20%2ATotal%20%C3%A0%20r%C3%A9gler%20%3A%2A%20%2A3150%20DH%2A%20%28dont%20arri%C3%A9r%C3%A9s%20%3A%201350%20DH%29%0A%0A%F0%9F%93%84%20%2AT%C3%A9l%C3%A9charger%20votre%20document%20officiel%20%28PDF%29%20%3A%2A%0A%F0%9F%91%89%20https%3A//srbl.netlify.app/pdf/appel-M02.pdf%0A%0A%F0%9F%8F%A6%20%2ACoordonn%C3%A9es%20bancaires%20pour%20le%20virement%20%3A%2A%0A%E2%80%A2%20%2AB%C3%A9n%C3%A9ficiaire%20%3A%2A%20SYNDICAT%20RESIDENCE%20BELLES%20LOGES%0A%E2%80%A2%20%2ABanque%20%3A%2A%20BMCE%20/%20BANK%20OF%20AFRICA%0A%E2%80%A2%20%2ARIB%20%3A%2A%20%60011%20780%200000402100011545%2025%60%0A%0A_Motif%20%3A%20M02%20-%20HIND%20DRIOUECH%20ET%20MR%20ABDELAH%20NACHIT_%0A%0AMerci%20pour%20votre%20pr%C3%A9cieuse%20collaboration.%0A%2ALe%20Bureau%20du%20Syndic%2A", "📲 Envoyer WhatsApp Direct")</f>
+        <v/>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>🏢 *SYNDICAT RÉSIDENCE BELLES LOGES*
+📍 Rue Attabari, Quartier Les Princesses, Casablanca
+Bonjour *HIND DRIOUECH ET MR ABDELAH NACHIT*,
+Veuillez trouver ci-dessous l'appel de cotisations syndicales pour votre bien (*Magasin N° 2* / M02) :
+📅 *Période :* Année 2026
+💰 *Total à régler :* *3150 DH* (dont arriérés : 1350 DH)
+📄 *Télécharger votre document officiel (PDF) :*
+👉 https://srbl.netlify.app/pdf/appel-M02.pdf
+🏦 *Coordonnées bancaires pour le virement :*
+• *Bénéficiaire :* SYNDICAT RESIDENCE BELLES LOGES
+• *Banque :* BMCE / BANK OF AFRICA
+• *RIB :* `011 780 0000402100011545 25`
+_Motif : M02 - HIND DRIOUECH ET MR ABDELAH NACHIT_
+Merci pour votre précieuse collaboration.
+*Le Bureau du Syndic*</t>
+        </is>
+      </c>
+      <c r="Z8" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/?client=M02", "👤 Espace Client (M02)")</f>
+        <v/>
+      </c>
     </row>
     <row r="9" ht="24.75" customHeight="1">
       <c r="B9" s="128" t="inlineStr">
@@ -3208,6 +3334,37 @@
       </c>
       <c r="V9" s="127">
         <f>'Cotisation 2025'!V9</f>
+        <v/>
+      </c>
+      <c r="W9" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/pdf/appel-M03.pdf", "📄 Voir PDF (M03)")</f>
+        <v/>
+      </c>
+      <c r="X9" s="268">
+        <f>HYPERLINK("https://wa.me/212669791313?text=%F0%9F%8F%A2%20%2ASYNDICAT%20R%C3%89SIDENCE%20BELLES%20LOGES%2A%0A%F0%9F%93%8D%20Rue%20Attabari%2C%20Quartier%20Les%20Princesses%2C%20Casablanca%0A%0ABonjour%20%2AHIND%20DRIOUECH%20ET%20MR%20ABDELAH%20NACHIT%2A%2C%0A%0AVeuillez%20trouver%20ci-dessous%20l%27appel%20de%20cotisations%20syndicales%20pour%20votre%20bien%20%28%2AMagasin%20N%C2%B0%203%2A%20/%20M03%29%20%3A%0A%0A%F0%9F%93%85%20%2AP%C3%A9riode%20%3A%2A%20Ann%C3%A9e%202026%0A%F0%9F%92%B0%20%2ATotal%20%C3%A0%20r%C3%A9gler%20%3A%2A%20%2A1800%20DH%2A%0A%0A%F0%9F%93%84%20%2AT%C3%A9l%C3%A9charger%20votre%20document%20officiel%20%28PDF%29%20%3A%2A%0A%F0%9F%91%89%20https%3A//srbl.netlify.app/pdf/appel-M03.pdf%0A%0A%F0%9F%8F%A6%20%2ACoordonn%C3%A9es%20bancaires%20pour%20le%20virement%20%3A%2A%0A%E2%80%A2%20%2AB%C3%A9n%C3%A9ficiaire%20%3A%2A%20SYNDICAT%20RESIDENCE%20BELLES%20LOGES%0A%E2%80%A2%20%2ABanque%20%3A%2A%20BMCE%20/%20BANK%20OF%20AFRICA%0A%E2%80%A2%20%2ARIB%20%3A%2A%20%60011%20780%200000402100011545%2025%60%0A%0A_Motif%20%3A%20M03%20-%20HIND%20DRIOUECH%20ET%20MR%20ABDELAH%20NACHIT_%0A%0AMerci%20pour%20votre%20pr%C3%A9cieuse%20collaboration.%0A%2ALe%20Bureau%20du%20Syndic%2A", "📲 Envoyer WhatsApp Direct")</f>
+        <v/>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>🏢 *SYNDICAT RÉSIDENCE BELLES LOGES*
+📍 Rue Attabari, Quartier Les Princesses, Casablanca
+Bonjour *HIND DRIOUECH ET MR ABDELAH NACHIT*,
+Veuillez trouver ci-dessous l'appel de cotisations syndicales pour votre bien (*Magasin N° 3* / M03) :
+📅 *Période :* Année 2026
+💰 *Total à régler :* *1800 DH*
+📄 *Télécharger votre document officiel (PDF) :*
+👉 https://srbl.netlify.app/pdf/appel-M03.pdf
+🏦 *Coordonnées bancaires pour le virement :*
+• *Bénéficiaire :* SYNDICAT RESIDENCE BELLES LOGES
+• *Banque :* BMCE / BANK OF AFRICA
+• *RIB :* `011 780 0000402100011545 25`
+_Motif : M03 - HIND DRIOUECH ET MR ABDELAH NACHIT_
+Merci pour votre précieuse collaboration.
+*Le Bureau du Syndic*</t>
+        </is>
+      </c>
+      <c r="Z9" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/?client=M03", "👤 Espace Client (M03)")</f>
         <v/>
       </c>
     </row>
@@ -3281,6 +3438,37 @@
         <f>'Cotisation 2025'!V10</f>
         <v/>
       </c>
+      <c r="W10" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/pdf/appel-M04.pdf", "📄 Voir PDF (M04)")</f>
+        <v/>
+      </c>
+      <c r="X10" s="268">
+        <f>HYPERLINK("https://wa.me/212669281802?text=%F0%9F%8F%A2%20%2ASYNDICAT%20R%C3%89SIDENCE%20BELLES%20LOGES%2A%0A%F0%9F%93%8D%20Rue%20Attabari%2C%20Quartier%20Les%20Princesses%2C%20Casablanca%0A%0ABonjour%20%2ANMJ%20CAPITAL%2A%2C%0A%0AVeuillez%20trouver%20ci-dessous%20l%27appel%20de%20cotisations%20syndicales%20pour%20votre%20bien%20%28%2AMagasin%20N%C2%B0%204%2A%20/%20M04%29%20%3A%0A%0A%F0%9F%93%85%20%2AP%C3%A9riode%20%3A%2A%20Ann%C3%A9e%202026%0A%F0%9F%92%B0%20%2ATotal%20%C3%A0%20r%C3%A9gler%20%3A%2A%20%2A1800%20DH%2A%0A%0A%F0%9F%93%84%20%2AT%C3%A9l%C3%A9charger%20votre%20document%20officiel%20%28PDF%29%20%3A%2A%0A%F0%9F%91%89%20https%3A//srbl.netlify.app/pdf/appel-M04.pdf%0A%0A%F0%9F%8F%A6%20%2ACoordonn%C3%A9es%20bancaires%20pour%20le%20virement%20%3A%2A%0A%E2%80%A2%20%2AB%C3%A9n%C3%A9ficiaire%20%3A%2A%20SYNDICAT%20RESIDENCE%20BELLES%20LOGES%0A%E2%80%A2%20%2ABanque%20%3A%2A%20BMCE%20/%20BANK%20OF%20AFRICA%0A%E2%80%A2%20%2ARIB%20%3A%2A%20%60011%20780%200000402100011545%2025%60%0A%0A_Motif%20%3A%20M04%20-%20NMJ%20CAPITAL_%0A%0AMerci%20pour%20votre%20pr%C3%A9cieuse%20collaboration.%0A%2ALe%20Bureau%20du%20Syndic%2A", "📲 Envoyer WhatsApp Direct")</f>
+        <v/>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>🏢 *SYNDICAT RÉSIDENCE BELLES LOGES*
+📍 Rue Attabari, Quartier Les Princesses, Casablanca
+Bonjour *NMJ CAPITAL*,
+Veuillez trouver ci-dessous l'appel de cotisations syndicales pour votre bien (*Magasin N° 4* / M04) :
+📅 *Période :* Année 2026
+💰 *Total à régler :* *1800 DH*
+📄 *Télécharger votre document officiel (PDF) :*
+👉 https://srbl.netlify.app/pdf/appel-M04.pdf
+🏦 *Coordonnées bancaires pour le virement :*
+• *Bénéficiaire :* SYNDICAT RESIDENCE BELLES LOGES
+• *Banque :* BMCE / BANK OF AFRICA
+• *RIB :* `011 780 0000402100011545 25`
+_Motif : M04 - NMJ CAPITAL_
+Merci pour votre précieuse collaboration.
+*Le Bureau du Syndic*</t>
+        </is>
+      </c>
+      <c r="Z10" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/?client=M04", "👤 Espace Client (M04)")</f>
+        <v/>
+      </c>
     </row>
     <row r="11" ht="24.95" customHeight="1">
       <c r="B11" s="131" t="inlineStr">
@@ -3332,13 +3520,13 @@
         <v>300</v>
       </c>
       <c r="P11" s="55" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="Q11" s="55" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="R11" s="55" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="S11" s="126">
         <f>SUM(G11:R11)</f>
@@ -3356,6 +3544,37 @@
         <f>'Cotisation 2025'!V11</f>
         <v/>
       </c>
+      <c r="W11" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/pdf/appel-A10.pdf", "📄 Voir PDF (A10)")</f>
+        <v/>
+      </c>
+      <c r="X11" s="268">
+        <f>HYPERLINK("https://wa.me/212662773532?text=%F0%9F%8F%A2%20%2ASYNDICAT%20R%C3%89SIDENCE%20BELLES%20LOGES%2A%0A%F0%9F%93%8D%20Rue%20Attabari%2C%20Quartier%20Les%20Princesses%2C%20Casablanca%0A%0ABonjour%20%2ABENYAHYA%20IHSAN%2A%2C%0A%0AVeuillez%20trouver%20ci-dessous%20l%27appel%20de%20cotisations%20syndicales%20pour%20votre%20bien%20%28%2AAppartement%20N%C2%B01%2A%20/%20A10%29%20%3A%0A%0A%F0%9F%93%85%20%2AP%C3%A9riode%20%3A%2A%20Ann%C3%A9e%202026%0A%F0%9F%92%B0%20%2ATotal%20%C3%A0%20r%C3%A9gler%20%3A%2A%20%2A3600%20DH%2A%0A%0A%F0%9F%93%84%20%2AT%C3%A9l%C3%A9charger%20votre%20document%20officiel%20%28PDF%29%20%3A%2A%0A%F0%9F%91%89%20https%3A//srbl.netlify.app/pdf/appel-A10.pdf%0A%0A%F0%9F%8F%A6%20%2ACoordonn%C3%A9es%20bancaires%20pour%20le%20virement%20%3A%2A%0A%E2%80%A2%20%2AB%C3%A9n%C3%A9ficiaire%20%3A%2A%20SYNDICAT%20RESIDENCE%20BELLES%20LOGES%0A%E2%80%A2%20%2ABanque%20%3A%2A%20BMCE%20/%20BANK%20OF%20AFRICA%0A%E2%80%A2%20%2ARIB%20%3A%2A%20%60011%20780%200000402100011545%2025%60%0A%0A_Motif%20%3A%20A10%20-%20BENYAHYA%20IHSAN_%0A%0AMerci%20pour%20votre%20pr%C3%A9cieuse%20collaboration.%0A%2ALe%20Bureau%20du%20Syndic%2A", "📲 Envoyer WhatsApp Direct")</f>
+        <v/>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>🏢 *SYNDICAT RÉSIDENCE BELLES LOGES*
+📍 Rue Attabari, Quartier Les Princesses, Casablanca
+Bonjour *BENYAHYA IHSAN*,
+Veuillez trouver ci-dessous l'appel de cotisations syndicales pour votre bien (*Appartement N°1* / A10) :
+📅 *Période :* Année 2026
+💰 *Total à régler :* *3600 DH*
+📄 *Télécharger votre document officiel (PDF) :*
+👉 https://srbl.netlify.app/pdf/appel-A10.pdf
+🏦 *Coordonnées bancaires pour le virement :*
+• *Bénéficiaire :* SYNDICAT RESIDENCE BELLES LOGES
+• *Banque :* BMCE / BANK OF AFRICA
+• *RIB :* `011 780 0000402100011545 25`
+_Motif : A10 - BENYAHYA IHSAN_
+Merci pour votre précieuse collaboration.
+*Le Bureau du Syndic*</t>
+        </is>
+      </c>
+      <c r="Z11" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/?client=A10", "👤 Espace Client (A10)")</f>
+        <v/>
+      </c>
     </row>
     <row r="12" ht="24.95" customHeight="1">
       <c r="B12" s="133" t="inlineStr">
@@ -3429,6 +3648,37 @@
         <f>'Cotisation 2025'!V12</f>
         <v/>
       </c>
+      <c r="W12" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/pdf/appel-A02.pdf", "📄 Voir PDF (A02)")</f>
+        <v/>
+      </c>
+      <c r="X12" s="268">
+        <f>HYPERLINK("https://wa.me/212661411823?text=%F0%9F%8F%A2%20%2ASYNDICAT%20R%C3%89SIDENCE%20BELLES%20LOGES%2A%0A%F0%9F%93%8D%20Rue%20Attabari%2C%20Quartier%20Les%20Princesses%2C%20Casablanca%0A%0ABonjour%20%2AGHALLAB%20HAKIM%2A%2C%0A%0AVeuillez%20trouver%20ci-dessous%20l%27appel%20de%20cotisations%20syndicales%20pour%20votre%20bien%20%28%2AAppartement%20N%C2%B02%2A%20/%20A02%29%20%3A%0A%0A%F0%9F%93%85%20%2AP%C3%A9riode%20%3A%2A%20Ann%C3%A9e%202026%0A%F0%9F%92%B0%20%2ATotal%20%C3%A0%20r%C3%A9gler%20%3A%2A%20%2A3600%20DH%2A%0A%0A%F0%9F%93%84%20%2AT%C3%A9l%C3%A9charger%20votre%20document%20officiel%20%28PDF%29%20%3A%2A%0A%F0%9F%91%89%20https%3A//srbl.netlify.app/pdf/appel-A02.pdf%0A%0A%F0%9F%8F%A6%20%2ACoordonn%C3%A9es%20bancaires%20pour%20le%20virement%20%3A%2A%0A%E2%80%A2%20%2AB%C3%A9n%C3%A9ficiaire%20%3A%2A%20SYNDICAT%20RESIDENCE%20BELLES%20LOGES%0A%E2%80%A2%20%2ABanque%20%3A%2A%20BMCE%20/%20BANK%20OF%20AFRICA%0A%E2%80%A2%20%2ARIB%20%3A%2A%20%60011%20780%200000402100011545%2025%60%0A%0A_Motif%20%3A%20A02%20-%20GHALLAB%20HAKIM_%0A%0AMerci%20pour%20votre%20pr%C3%A9cieuse%20collaboration.%0A%2ALe%20Bureau%20du%20Syndic%2A", "📲 Envoyer WhatsApp Direct")</f>
+        <v/>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>🏢 *SYNDICAT RÉSIDENCE BELLES LOGES*
+📍 Rue Attabari, Quartier Les Princesses, Casablanca
+Bonjour *GHALLAB HAKIM*,
+Veuillez trouver ci-dessous l'appel de cotisations syndicales pour votre bien (*Appartement N°2* / A02) :
+📅 *Période :* Année 2026
+💰 *Total à régler :* *3600 DH*
+📄 *Télécharger votre document officiel (PDF) :*
+👉 https://srbl.netlify.app/pdf/appel-A02.pdf
+🏦 *Coordonnées bancaires pour le virement :*
+• *Bénéficiaire :* SYNDICAT RESIDENCE BELLES LOGES
+• *Banque :* BMCE / BANK OF AFRICA
+• *RIB :* `011 780 0000402100011545 25`
+_Motif : A02 - GHALLAB HAKIM_
+Merci pour votre précieuse collaboration.
+*Le Bureau du Syndic*</t>
+        </is>
+      </c>
+      <c r="Z12" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/?client=A02", "👤 Espace Client (A02)")</f>
+        <v/>
+      </c>
     </row>
     <row r="13" ht="28.15" customHeight="1">
       <c r="B13" s="128" t="inlineStr">
@@ -3502,6 +3752,37 @@
         <f>'Cotisation 2025'!V13</f>
         <v/>
       </c>
+      <c r="W13" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/pdf/appel-A03.pdf", "📄 Voir PDF (A03)")</f>
+        <v/>
+      </c>
+      <c r="X13" s="268">
+        <f>HYPERLINK("https://wa.me/212619082870?text=%F0%9F%8F%A2%20%2ASYNDICAT%20R%C3%89SIDENCE%20BELLES%20LOGES%2A%0A%F0%9F%93%8D%20Rue%20Attabari%2C%20Quartier%20Les%20Princesses%2C%20Casablanca%0A%0ABonjour%20%2ANADIL%20IMANE%2A%2C%0A%0AVeuillez%20trouver%20ci-dessous%20l%27appel%20de%20cotisations%20syndicales%20pour%20votre%20bien%20%28%2AAppartement%20N%C2%B03%2A%20/%20A03%29%20%3A%0A%0A%F0%9F%93%85%20%2AP%C3%A9riode%20%3A%2A%20Ann%C3%A9e%202026%0A%F0%9F%92%B0%20%2ATotal%20%C3%A0%20r%C3%A9gler%20%3A%2A%20%2A3600%20DH%2A%0A%0A%F0%9F%93%84%20%2AT%C3%A9l%C3%A9charger%20votre%20document%20officiel%20%28PDF%29%20%3A%2A%0A%F0%9F%91%89%20https%3A//srbl.netlify.app/pdf/appel-A03.pdf%0A%0A%F0%9F%8F%A6%20%2ACoordonn%C3%A9es%20bancaires%20pour%20le%20virement%20%3A%2A%0A%E2%80%A2%20%2AB%C3%A9n%C3%A9ficiaire%20%3A%2A%20SYNDICAT%20RESIDENCE%20BELLES%20LOGES%0A%E2%80%A2%20%2ABanque%20%3A%2A%20BMCE%20/%20BANK%20OF%20AFRICA%0A%E2%80%A2%20%2ARIB%20%3A%2A%20%60011%20780%200000402100011545%2025%60%0A%0A_Motif%20%3A%20A03%20-%20NADIL%20IMANE_%0A%0AMerci%20pour%20votre%20pr%C3%A9cieuse%20collaboration.%0A%2ALe%20Bureau%20du%20Syndic%2A", "📲 Envoyer WhatsApp Direct")</f>
+        <v/>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>🏢 *SYNDICAT RÉSIDENCE BELLES LOGES*
+📍 Rue Attabari, Quartier Les Princesses, Casablanca
+Bonjour *NADIL IMANE*,
+Veuillez trouver ci-dessous l'appel de cotisations syndicales pour votre bien (*Appartement N°3* / A03) :
+📅 *Période :* Année 2026
+💰 *Total à régler :* *3600 DH*
+📄 *Télécharger votre document officiel (PDF) :*
+👉 https://srbl.netlify.app/pdf/appel-A03.pdf
+🏦 *Coordonnées bancaires pour le virement :*
+• *Bénéficiaire :* SYNDICAT RESIDENCE BELLES LOGES
+• *Banque :* BMCE / BANK OF AFRICA
+• *RIB :* `011 780 0000402100011545 25`
+_Motif : A03 - NADIL IMANE_
+Merci pour votre précieuse collaboration.
+*Le Bureau du Syndic*</t>
+        </is>
+      </c>
+      <c r="Z13" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/?client=A03", "👤 Espace Client (A03)")</f>
+        <v/>
+      </c>
     </row>
     <row r="14" ht="27.6" customHeight="1">
       <c r="B14" s="128" t="inlineStr">
@@ -3575,6 +3856,37 @@
         <f>'Cotisation 2025'!V14</f>
         <v/>
       </c>
+      <c r="W14" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/pdf/appel-A04.pdf", "📄 Voir PDF (A04)")</f>
+        <v/>
+      </c>
+      <c r="X14" s="268">
+        <f>HYPERLINK("https://wa.me/212661377432?text=%F0%9F%8F%A2%20%2ASYNDICAT%20R%C3%89SIDENCE%20BELLES%20LOGES%2A%0A%F0%9F%93%8D%20Rue%20Attabari%2C%20Quartier%20Les%20Princesses%2C%20Casablanca%0A%0ABonjour%20%2AINSAF%20BASSIL%2A%2C%0A%0AVeuillez%20trouver%20ci-dessous%20l%27appel%20de%20cotisations%20syndicales%20pour%20votre%20bien%20%28%2AAppartement%20N%C2%B04%2A%20/%20A04%29%20%3A%0A%0A%F0%9F%93%85%20%2AP%C3%A9riode%20%3A%2A%20Ann%C3%A9e%202026%0A%F0%9F%92%B0%20%2ATotal%20%C3%A0%20r%C3%A9gler%20%3A%2A%20%2A5250%20DH%2A%20%28dont%20arri%C3%A9r%C3%A9s%20%3A%201650%20DH%29%0A%0A%F0%9F%93%84%20%2AT%C3%A9l%C3%A9charger%20votre%20document%20officiel%20%28PDF%29%20%3A%2A%0A%F0%9F%91%89%20https%3A//srbl.netlify.app/pdf/appel-A04.pdf%0A%0A%F0%9F%8F%A6%20%2ACoordonn%C3%A9es%20bancaires%20pour%20le%20virement%20%3A%2A%0A%E2%80%A2%20%2AB%C3%A9n%C3%A9ficiaire%20%3A%2A%20SYNDICAT%20RESIDENCE%20BELLES%20LOGES%0A%E2%80%A2%20%2ABanque%20%3A%2A%20BMCE%20/%20BANK%20OF%20AFRICA%0A%E2%80%A2%20%2ARIB%20%3A%2A%20%60011%20780%200000402100011545%2025%60%0A%0A_Motif%20%3A%20A04%20-%20INSAF%20BASSIL_%0A%0AMerci%20pour%20votre%20pr%C3%A9cieuse%20collaboration.%0A%2ALe%20Bureau%20du%20Syndic%2A", "📲 Envoyer WhatsApp Direct")</f>
+        <v/>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>🏢 *SYNDICAT RÉSIDENCE BELLES LOGES*
+📍 Rue Attabari, Quartier Les Princesses, Casablanca
+Bonjour *INSAF BASSIL*,
+Veuillez trouver ci-dessous l'appel de cotisations syndicales pour votre bien (*Appartement N°4* / A04) :
+📅 *Période :* Année 2026
+💰 *Total à régler :* *5250 DH* (dont arriérés : 1650 DH)
+📄 *Télécharger votre document officiel (PDF) :*
+👉 https://srbl.netlify.app/pdf/appel-A04.pdf
+🏦 *Coordonnées bancaires pour le virement :*
+• *Bénéficiaire :* SYNDICAT RESIDENCE BELLES LOGES
+• *Banque :* BMCE / BANK OF AFRICA
+• *RIB :* `011 780 0000402100011545 25`
+_Motif : A04 - INSAF BASSIL_
+Merci pour votre précieuse collaboration.
+*Le Bureau du Syndic*</t>
+        </is>
+      </c>
+      <c r="Z14" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/?client=A04", "👤 Espace Client (A04)")</f>
+        <v/>
+      </c>
     </row>
     <row r="15" ht="24.6" customHeight="1">
       <c r="B15" s="135" t="inlineStr">
@@ -3648,6 +3960,37 @@
         <f>'Cotisation 2025'!V15</f>
         <v/>
       </c>
+      <c r="W15" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/pdf/appel-A05.pdf", "📄 Voir PDF (A05)")</f>
+        <v/>
+      </c>
+      <c r="X15" s="268">
+        <f>HYPERLINK("https://wa.me/447551433285?text=%F0%9F%8F%A2%20%2ASYNDICAT%20R%C3%89SIDENCE%20BELLES%20LOGES%2A%0A%F0%9F%93%8D%20Rue%20Attabari%2C%20Quartier%20Les%20Princesses%2C%20Casablanca%0A%0ABonjour%20%2AMME%20TORRES%20HIND%2A%2C%0A%0AVeuillez%20trouver%20ci-dessous%20l%27appel%20de%20cotisations%20syndicales%20pour%20votre%20bien%20%28%2AAppartement%20N%C2%B05%2A%20/%20A05%29%20%3A%0A%0A%F0%9F%93%85%20%2AP%C3%A9riode%20%3A%2A%20Ann%C3%A9e%202026%0A%F0%9F%92%B0%20%2ATotal%20%C3%A0%20r%C3%A9gler%20%3A%2A%20%2A3600%20DH%2A%0A%0A%F0%9F%93%84%20%2AT%C3%A9l%C3%A9charger%20votre%20document%20officiel%20%28PDF%29%20%3A%2A%0A%F0%9F%91%89%20https%3A//srbl.netlify.app/pdf/appel-A05.pdf%0A%0A%F0%9F%8F%A6%20%2ACoordonn%C3%A9es%20bancaires%20pour%20le%20virement%20%3A%2A%0A%E2%80%A2%20%2AB%C3%A9n%C3%A9ficiaire%20%3A%2A%20SYNDICAT%20RESIDENCE%20BELLES%20LOGES%0A%E2%80%A2%20%2ABanque%20%3A%2A%20BMCE%20/%20BANK%20OF%20AFRICA%0A%E2%80%A2%20%2ARIB%20%3A%2A%20%60011%20780%200000402100011545%2025%60%0A%0A_Motif%20%3A%20A05%20-%20MME%20TORRES%20HIND_%0A%0AMerci%20pour%20votre%20pr%C3%A9cieuse%20collaboration.%0A%2ALe%20Bureau%20du%20Syndic%2A", "📲 Envoyer WhatsApp Direct")</f>
+        <v/>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>🏢 *SYNDICAT RÉSIDENCE BELLES LOGES*
+📍 Rue Attabari, Quartier Les Princesses, Casablanca
+Bonjour *MME TORRES HIND*,
+Veuillez trouver ci-dessous l'appel de cotisations syndicales pour votre bien (*Appartement N°5* / A05) :
+📅 *Période :* Année 2026
+💰 *Total à régler :* *3600 DH*
+📄 *Télécharger votre document officiel (PDF) :*
+👉 https://srbl.netlify.app/pdf/appel-A05.pdf
+🏦 *Coordonnées bancaires pour le virement :*
+• *Bénéficiaire :* SYNDICAT RESIDENCE BELLES LOGES
+• *Banque :* BMCE / BANK OF AFRICA
+• *RIB :* `011 780 0000402100011545 25`
+_Motif : A05 - MME TORRES HIND_
+Merci pour votre précieuse collaboration.
+*Le Bureau du Syndic*</t>
+        </is>
+      </c>
+      <c r="Z15" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/?client=A05", "👤 Espace Client (A05)")</f>
+        <v/>
+      </c>
     </row>
     <row r="16" ht="24.95" customHeight="1">
       <c r="B16" s="136" t="inlineStr">
@@ -3721,6 +4064,37 @@
         <f>'Cotisation 2025'!V16</f>
         <v/>
       </c>
+      <c r="W16" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/pdf/appel-A06.pdf", "📄 Voir PDF (A06)")</f>
+        <v/>
+      </c>
+      <c r="X16" s="268">
+        <f>HYPERLINK("https://wa.me/212669281802?text=%F0%9F%8F%A2%20%2ASYNDICAT%20R%C3%89SIDENCE%20BELLES%20LOGES%2A%0A%F0%9F%93%8D%20Rue%20Attabari%2C%20Quartier%20Les%20Princesses%2C%20Casablanca%0A%0ABonjour%20%2ANMJ%20CAPITAL%20/%20BEN%20HADDOUCH%20YOUNES%2A%2C%0A%0AVeuillez%20trouver%20ci-dessous%20l%27appel%20de%20cotisations%20syndicales%20pour%20votre%20bien%20%28%2AAppartement%20N%C2%B06%2A%20/%20A06%29%20%3A%0A%0A%F0%9F%93%85%20%2AP%C3%A9riode%20%3A%2A%20Ann%C3%A9e%202026%0A%F0%9F%92%B0%20%2ATotal%20%C3%A0%20r%C3%A9gler%20%3A%2A%20%2A4800%20DH%2A%20%28dont%20arri%C3%A9r%C3%A9s%20%3A%201200%20DH%29%0A%0A%F0%9F%93%84%20%2AT%C3%A9l%C3%A9charger%20votre%20document%20officiel%20%28PDF%29%20%3A%2A%0A%F0%9F%91%89%20https%3A//srbl.netlify.app/pdf/appel-A06.pdf%0A%0A%F0%9F%8F%A6%20%2ACoordonn%C3%A9es%20bancaires%20pour%20le%20virement%20%3A%2A%0A%E2%80%A2%20%2AB%C3%A9n%C3%A9ficiaire%20%3A%2A%20SYNDICAT%20RESIDENCE%20BELLES%20LOGES%0A%E2%80%A2%20%2ABanque%20%3A%2A%20BMCE%20/%20BANK%20OF%20AFRICA%0A%E2%80%A2%20%2ARIB%20%3A%2A%20%60011%20780%200000402100011545%2025%60%0A%0A_Motif%20%3A%20A06%20-%20NMJ%20CAPITAL%20/%20BEN%20HADDOUCH%20YOUNES_%0A%0AMerci%20pour%20votre%20pr%C3%A9cieuse%20collaboration.%0A%2ALe%20Bureau%20du%20Syndic%2A", "📲 Envoyer WhatsApp Direct")</f>
+        <v/>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>🏢 *SYNDICAT RÉSIDENCE BELLES LOGES*
+📍 Rue Attabari, Quartier Les Princesses, Casablanca
+Bonjour *NMJ CAPITAL / BEN HADDOUCH YOUNES*,
+Veuillez trouver ci-dessous l'appel de cotisations syndicales pour votre bien (*Appartement N°6* / A06) :
+📅 *Période :* Année 2026
+💰 *Total à régler :* *4800 DH* (dont arriérés : 1200 DH)
+📄 *Télécharger votre document officiel (PDF) :*
+👉 https://srbl.netlify.app/pdf/appel-A06.pdf
+🏦 *Coordonnées bancaires pour le virement :*
+• *Bénéficiaire :* SYNDICAT RESIDENCE BELLES LOGES
+• *Banque :* BMCE / BANK OF AFRICA
+• *RIB :* `011 780 0000402100011545 25`
+_Motif : A06 - NMJ CAPITAL / BEN HADDOUCH YOUNES_
+Merci pour votre précieuse collaboration.
+*Le Bureau du Syndic*</t>
+        </is>
+      </c>
+      <c r="Z16" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/?client=A06", "👤 Espace Client (A06)")</f>
+        <v/>
+      </c>
     </row>
     <row r="17" ht="24.95" customHeight="1">
       <c r="B17" s="131" t="inlineStr">
@@ -3796,6 +4170,37 @@
         <f>'Cotisation 2025'!V17</f>
         <v/>
       </c>
+      <c r="W17" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/pdf/appel-A07.pdf", "📄 Voir PDF (A07)")</f>
+        <v/>
+      </c>
+      <c r="X17" s="268">
+        <f>HYPERLINK("https://wa.me/212662773532?text=%F0%9F%8F%A2%20%2ASYNDICAT%20R%C3%89SIDENCE%20BELLES%20LOGES%2A%0A%F0%9F%93%8D%20Rue%20Attabari%2C%20Quartier%20Les%20Princesses%2C%20Casablanca%0A%0ABonjour%20%2ABENYAHYA%20IHSAN%2A%2C%0A%0AVeuillez%20trouver%20ci-dessous%20l%27appel%20de%20cotisations%20syndicales%20pour%20votre%20bien%20%28%2AAppartement%20N%C2%B07%2A%20/%20A07%29%20%3A%0A%0A%F0%9F%93%85%20%2AP%C3%A9riode%20%3A%2A%20Ann%C3%A9e%202026%0A%F0%9F%92%B0%20%2ATotal%20%C3%A0%20r%C3%A9gler%20%3A%2A%20%2A3600%20DH%2A%0A%0A%F0%9F%93%84%20%2AT%C3%A9l%C3%A9charger%20votre%20document%20officiel%20%28PDF%29%20%3A%2A%0A%F0%9F%91%89%20https%3A//srbl.netlify.app/pdf/appel-A07.pdf%0A%0A%F0%9F%8F%A6%20%2ACoordonn%C3%A9es%20bancaires%20pour%20le%20virement%20%3A%2A%0A%E2%80%A2%20%2AB%C3%A9n%C3%A9ficiaire%20%3A%2A%20SYNDICAT%20RESIDENCE%20BELLES%20LOGES%0A%E2%80%A2%20%2ABanque%20%3A%2A%20BMCE%20/%20BANK%20OF%20AFRICA%0A%E2%80%A2%20%2ARIB%20%3A%2A%20%60011%20780%200000402100011545%2025%60%0A%0A_Motif%20%3A%20A07%20-%20BENYAHYA%20IHSAN_%0A%0AMerci%20pour%20votre%20pr%C3%A9cieuse%20collaboration.%0A%2ALe%20Bureau%20du%20Syndic%2A", "📲 Envoyer WhatsApp Direct")</f>
+        <v/>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>🏢 *SYNDICAT RÉSIDENCE BELLES LOGES*
+📍 Rue Attabari, Quartier Les Princesses, Casablanca
+Bonjour *BENYAHYA IHSAN*,
+Veuillez trouver ci-dessous l'appel de cotisations syndicales pour votre bien (*Appartement N°7* / A07) :
+📅 *Période :* Année 2026
+💰 *Total à régler :* *3600 DH*
+📄 *Télécharger votre document officiel (PDF) :*
+👉 https://srbl.netlify.app/pdf/appel-A07.pdf
+🏦 *Coordonnées bancaires pour le virement :*
+• *Bénéficiaire :* SYNDICAT RESIDENCE BELLES LOGES
+• *Banque :* BMCE / BANK OF AFRICA
+• *RIB :* `011 780 0000402100011545 25`
+_Motif : A07 - BENYAHYA IHSAN_
+Merci pour votre précieuse collaboration.
+*Le Bureau du Syndic*</t>
+        </is>
+      </c>
+      <c r="Z17" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/?client=A07", "👤 Espace Client (A07)")</f>
+        <v/>
+      </c>
     </row>
     <row r="18" ht="24.75" customHeight="1">
       <c r="A18" t="inlineStr">
@@ -3874,6 +4279,37 @@
         <f>'Cotisation 2025'!V18</f>
         <v/>
       </c>
+      <c r="W18" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/pdf/appel-A08.pdf", "📄 Voir PDF (A08)")</f>
+        <v/>
+      </c>
+      <c r="X18" s="268">
+        <f>HYPERLINK("https://wa.me/212661286870?text=%F0%9F%8F%A2%20%2ASYNDICAT%20R%C3%89SIDENCE%20BELLES%20LOGES%2A%0A%F0%9F%93%8D%20Rue%20Attabari%2C%20Quartier%20Les%20Princesses%2C%20Casablanca%0A%0ABonjour%20%2AMR%20LAHBABI%20NIZAR%20%28COR%2A%2C%0A%0AVeuillez%20trouver%20ci-dessous%20l%27appel%20de%20cotisations%20syndicales%20pour%20votre%20bien%20%28%2AAppartement%20N%C2%B08%2A%20/%20A08%29%20%3A%0A%0A%F0%9F%93%85%20%2AP%C3%A9riode%20%3A%2A%20Ann%C3%A9e%202026%0A%F0%9F%92%B0%20%2ATotal%20%C3%A0%20r%C3%A9gler%20%3A%2A%20%2A3600%20DH%2A%0A%0A%F0%9F%93%84%20%2AT%C3%A9l%C3%A9charger%20votre%20document%20officiel%20%28PDF%29%20%3A%2A%0A%F0%9F%91%89%20https%3A//srbl.netlify.app/pdf/appel-A08.pdf%0A%0A%F0%9F%8F%A6%20%2ACoordonn%C3%A9es%20bancaires%20pour%20le%20virement%20%3A%2A%0A%E2%80%A2%20%2AB%C3%A9n%C3%A9ficiaire%20%3A%2A%20SYNDICAT%20RESIDENCE%20BELLES%20LOGES%0A%E2%80%A2%20%2ABanque%20%3A%2A%20BMCE%20/%20BANK%20OF%20AFRICA%0A%E2%80%A2%20%2ARIB%20%3A%2A%20%60011%20780%200000402100011545%2025%60%0A%0A_Motif%20%3A%20A08%20-%20MR%20LAHBABI%20NIZAR%20%28COR_%0A%0AMerci%20pour%20votre%20pr%C3%A9cieuse%20collaboration.%0A%2ALe%20Bureau%20du%20Syndic%2A", "📲 Envoyer WhatsApp Direct")</f>
+        <v/>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>🏢 *SYNDICAT RÉSIDENCE BELLES LOGES*
+📍 Rue Attabari, Quartier Les Princesses, Casablanca
+Bonjour *MR LAHBABI NIZAR (COR*,
+Veuillez trouver ci-dessous l'appel de cotisations syndicales pour votre bien (*Appartement N°8* / A08) :
+📅 *Période :* Année 2026
+💰 *Total à régler :* *3600 DH*
+📄 *Télécharger votre document officiel (PDF) :*
+👉 https://srbl.netlify.app/pdf/appel-A08.pdf
+🏦 *Coordonnées bancaires pour le virement :*
+• *Bénéficiaire :* SYNDICAT RESIDENCE BELLES LOGES
+• *Banque :* BMCE / BANK OF AFRICA
+• *RIB :* `011 780 0000402100011545 25`
+_Motif : A08 - MR LAHBABI NIZAR (COR_
+Merci pour votre précieuse collaboration.
+*Le Bureau du Syndic*</t>
+        </is>
+      </c>
+      <c r="Z18" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/?client=A08", "👤 Espace Client (A08)")</f>
+        <v/>
+      </c>
     </row>
     <row r="19" ht="24.95" customHeight="1">
       <c r="B19" s="128" t="inlineStr">
@@ -3947,6 +4383,37 @@
         <f>'Cotisation 2025'!V19</f>
         <v/>
       </c>
+      <c r="W19" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/pdf/appel-A09.pdf", "📄 Voir PDF (A09)")</f>
+        <v/>
+      </c>
+      <c r="X19" s="268">
+        <f>HYPERLINK("https://wa.me/212661936094?text=%F0%9F%8F%A2%20%2ASYNDICAT%20R%C3%89SIDENCE%20BELLES%20LOGES%2A%0A%F0%9F%93%8D%20Rue%20Attabari%2C%20Quartier%20Les%20Princesses%2C%20Casablanca%0A%0ABonjour%20%2AASRAGUIS%20ABDELGHANI%2A%2C%0A%0AVeuillez%20trouver%20ci-dessous%20l%27appel%20de%20cotisations%20syndicales%20pour%20votre%20bien%20%28%2AAppartement%20N%C2%B09%2A%20/%20A09%29%20%3A%0A%0A%F0%9F%93%85%20%2AP%C3%A9riode%20%3A%2A%20Ann%C3%A9e%202026%0A%F0%9F%92%B0%20%2ATotal%20%C3%A0%20r%C3%A9gler%20%3A%2A%20%2A3600%20DH%2A%0A%0A%F0%9F%93%84%20%2AT%C3%A9l%C3%A9charger%20votre%20document%20officiel%20%28PDF%29%20%3A%2A%0A%F0%9F%91%89%20https%3A//srbl.netlify.app/pdf/appel-A09.pdf%0A%0A%F0%9F%8F%A6%20%2ACoordonn%C3%A9es%20bancaires%20pour%20le%20virement%20%3A%2A%0A%E2%80%A2%20%2AB%C3%A9n%C3%A9ficiaire%20%3A%2A%20SYNDICAT%20RESIDENCE%20BELLES%20LOGES%0A%E2%80%A2%20%2ABanque%20%3A%2A%20BMCE%20/%20BANK%20OF%20AFRICA%0A%E2%80%A2%20%2ARIB%20%3A%2A%20%60011%20780%200000402100011545%2025%60%0A%0A_Motif%20%3A%20A09%20-%20ASRAGUIS%20ABDELGHANI_%0A%0AMerci%20pour%20votre%20pr%C3%A9cieuse%20collaboration.%0A%2ALe%20Bureau%20du%20Syndic%2A", "📲 Envoyer WhatsApp Direct")</f>
+        <v/>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>🏢 *SYNDICAT RÉSIDENCE BELLES LOGES*
+📍 Rue Attabari, Quartier Les Princesses, Casablanca
+Bonjour *ASRAGUIS ABDELGHANI*,
+Veuillez trouver ci-dessous l'appel de cotisations syndicales pour votre bien (*Appartement N°9* / A09) :
+📅 *Période :* Année 2026
+💰 *Total à régler :* *3600 DH*
+📄 *Télécharger votre document officiel (PDF) :*
+👉 https://srbl.netlify.app/pdf/appel-A09.pdf
+🏦 *Coordonnées bancaires pour le virement :*
+• *Bénéficiaire :* SYNDICAT RESIDENCE BELLES LOGES
+• *Banque :* BMCE / BANK OF AFRICA
+• *RIB :* `011 780 0000402100011545 25`
+_Motif : A09 - ASRAGUIS ABDELGHANI_
+Merci pour votre précieuse collaboration.
+*Le Bureau du Syndic*</t>
+        </is>
+      </c>
+      <c r="Z19" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/?client=A09", "👤 Espace Client (A09)")</f>
+        <v/>
+      </c>
     </row>
     <row r="20" ht="24.95" customHeight="1">
       <c r="B20" s="137" t="inlineStr">
@@ -3996,13 +4463,13 @@
         <v>300</v>
       </c>
       <c r="P20" s="55" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="Q20" s="55" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="R20" s="55" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="S20" s="126">
         <f>SUM(G20:R20)</f>
@@ -4020,6 +4487,37 @@
         <f>'Cotisation 2025'!V20</f>
         <v/>
       </c>
+      <c r="W20" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/pdf/appel-A10.pdf", "📄 Voir PDF (A10)")</f>
+        <v/>
+      </c>
+      <c r="X20" s="268">
+        <f>HYPERLINK("https://wa.me/212661157305?text=%F0%9F%8F%A2%20%2ASYNDICAT%20R%C3%89SIDENCE%20BELLES%20LOGES%2A%0A%F0%9F%93%8D%20Rue%20Attabari%2C%20Quartier%20Les%20Princesses%2C%20Casablanca%0A%0ABonjour%20%2AGHALLAB%20MOUHSSINE%2A%2C%0A%0AVeuillez%20trouver%20ci-dessous%20l%27appel%20de%20cotisations%20syndicales%20pour%20votre%20bien%20%28%2AAppartement%20N%C2%B010%2A%20/%20A10%29%20%3A%0A%0A%F0%9F%93%85%20%2AP%C3%A9riode%20%3A%2A%20Ann%C3%A9e%202026%0A%F0%9F%92%B0%20%2ATotal%20%C3%A0%20r%C3%A9gler%20%3A%2A%20%2A3600%20DH%2A%0A%0A%F0%9F%93%84%20%2AT%C3%A9l%C3%A9charger%20votre%20document%20officiel%20%28PDF%29%20%3A%2A%0A%F0%9F%91%89%20https%3A//srbl.netlify.app/pdf/appel-A10.pdf%0A%0A%F0%9F%8F%A6%20%2ACoordonn%C3%A9es%20bancaires%20pour%20le%20virement%20%3A%2A%0A%E2%80%A2%20%2AB%C3%A9n%C3%A9ficiaire%20%3A%2A%20SYNDICAT%20RESIDENCE%20BELLES%20LOGES%0A%E2%80%A2%20%2ABanque%20%3A%2A%20BMCE%20/%20BANK%20OF%20AFRICA%0A%E2%80%A2%20%2ARIB%20%3A%2A%20%60011%20780%200000402100011545%2025%60%0A%0A_Motif%20%3A%20A10%20-%20GHALLAB%20MOUHSSINE_%0A%0AMerci%20pour%20votre%20pr%C3%A9cieuse%20collaboration.%0A%2ALe%20Bureau%20du%20Syndic%2A", "📲 Envoyer WhatsApp Direct")</f>
+        <v/>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>🏢 *SYNDICAT RÉSIDENCE BELLES LOGES*
+📍 Rue Attabari, Quartier Les Princesses, Casablanca
+Bonjour *GHALLAB MOUHSSINE*,
+Veuillez trouver ci-dessous l'appel de cotisations syndicales pour votre bien (*Appartement N°10* / A10) :
+📅 *Période :* Année 2026
+💰 *Total à régler :* *3600 DH*
+📄 *Télécharger votre document officiel (PDF) :*
+👉 https://srbl.netlify.app/pdf/appel-A10.pdf
+🏦 *Coordonnées bancaires pour le virement :*
+• *Bénéficiaire :* SYNDICAT RESIDENCE BELLES LOGES
+• *Banque :* BMCE / BANK OF AFRICA
+• *RIB :* `011 780 0000402100011545 25`
+_Motif : A10 - GHALLAB MOUHSSINE_
+Merci pour votre précieuse collaboration.
+*Le Bureau du Syndic*</t>
+        </is>
+      </c>
+      <c r="Z20" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/?client=A10", "👤 Espace Client (A10)")</f>
+        <v/>
+      </c>
     </row>
     <row r="21" ht="24.95" customHeight="1">
       <c r="B21" s="135" t="inlineStr">
@@ -4060,22 +4558,22 @@
         <v>300</v>
       </c>
       <c r="M21" s="55" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="N21" s="55" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="O21" s="55" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="P21" s="55" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="Q21" s="55" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="R21" s="55" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="S21" s="126">
         <f>SUM(G21:R21)</f>
@@ -4093,6 +4591,37 @@
         <f>'Cotisation 2025'!V21</f>
         <v/>
       </c>
+      <c r="W21" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/pdf/appel-A11.pdf", "📄 Voir PDF (A11)")</f>
+        <v/>
+      </c>
+      <c r="X21" s="268">
+        <f>HYPERLINK("https://wa.me/447551433285?text=%F0%9F%8F%A2%20%2ASYNDICAT%20R%C3%89SIDENCE%20BELLES%20LOGES%2A%0A%F0%9F%93%8D%20Rue%20Attabari%2C%20Quartier%20Les%20Princesses%2C%20Casablanca%0A%0ABonjour%20%2AMME%20TORRES%20HIND%2A%2C%0A%0AVeuillez%20trouver%20ci-dessous%20l%27appel%20de%20cotisations%20syndicales%20pour%20votre%20bien%20%28%2AAppartement%20N%C2%B011%2A%20/%20A11%29%20%3A%0A%0A%F0%9F%93%85%20%2AP%C3%A9riode%20%3A%2A%20Ann%C3%A9e%202026%0A%F0%9F%92%B0%20%2ATotal%20%C3%A0%20r%C3%A9gler%20%3A%2A%20%2A3600%20DH%2A%0A%0A%F0%9F%93%84%20%2AT%C3%A9l%C3%A9charger%20votre%20document%20officiel%20%28PDF%29%20%3A%2A%0A%F0%9F%91%89%20https%3A//srbl.netlify.app/pdf/appel-A11.pdf%0A%0A%F0%9F%8F%A6%20%2ACoordonn%C3%A9es%20bancaires%20pour%20le%20virement%20%3A%2A%0A%E2%80%A2%20%2AB%C3%A9n%C3%A9ficiaire%20%3A%2A%20SYNDICAT%20RESIDENCE%20BELLES%20LOGES%0A%E2%80%A2%20%2ABanque%20%3A%2A%20BMCE%20/%20BANK%20OF%20AFRICA%0A%E2%80%A2%20%2ARIB%20%3A%2A%20%60011%20780%200000402100011545%2025%60%0A%0A_Motif%20%3A%20A11%20-%20MME%20TORRES%20HIND_%0A%0AMerci%20pour%20votre%20pr%C3%A9cieuse%20collaboration.%0A%2ALe%20Bureau%20du%20Syndic%2A", "📲 Envoyer WhatsApp Direct")</f>
+        <v/>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>🏢 *SYNDICAT RÉSIDENCE BELLES LOGES*
+📍 Rue Attabari, Quartier Les Princesses, Casablanca
+Bonjour *MME TORRES HIND*,
+Veuillez trouver ci-dessous l'appel de cotisations syndicales pour votre bien (*Appartement N°11* / A11) :
+📅 *Période :* Année 2026
+💰 *Total à régler :* *3600 DH*
+📄 *Télécharger votre document officiel (PDF) :*
+👉 https://srbl.netlify.app/pdf/appel-A11.pdf
+🏦 *Coordonnées bancaires pour le virement :*
+• *Bénéficiaire :* SYNDICAT RESIDENCE BELLES LOGES
+• *Banque :* BMCE / BANK OF AFRICA
+• *RIB :* `011 780 0000402100011545 25`
+_Motif : A11 - MME TORRES HIND_
+Merci pour votre précieuse collaboration.
+*Le Bureau du Syndic*</t>
+        </is>
+      </c>
+      <c r="Z21" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/?client=A11", "👤 Espace Client (A11)")</f>
+        <v/>
+      </c>
     </row>
     <row r="22" ht="24" customHeight="1">
       <c r="B22" s="172" t="inlineStr">
@@ -4115,7 +4644,7 @@
         </is>
       </c>
       <c r="G22" s="55" t="n">
-        <v>300</v>
+        <v>900</v>
       </c>
       <c r="H22" s="55" t="n">
         <v>300</v>
@@ -4166,6 +4695,37 @@
         <f>'Cotisation 2025'!V22</f>
         <v/>
       </c>
+      <c r="W22" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/pdf/appel-A01.pdf", "📄 Voir PDF (A01)")</f>
+        <v/>
+      </c>
+      <c r="X22" s="268">
+        <f>HYPERLINK("https://wa.me/212705262264?text=%F0%9F%8F%A2%20%2ASYNDICAT%20R%C3%89SIDENCE%20BELLES%20LOGES%2A%0A%F0%9F%93%8D%20Rue%20Attabari%2C%20Quartier%20Les%20Princesses%2C%20Casablanca%0A%0ABonjour%20%2AELMOSTAFA%20EL%20GUESSAB%2A%2C%0A%0AVeuillez%20trouver%20ci-dessous%20l%27appel%20de%20cotisations%20syndicales%20pour%20votre%20bien%20%28%2AAppartement%20N%C2%B012%2A%20/%20A01%29%20%3A%0A%0A%F0%9F%93%85%20%2AP%C3%A9riode%20%3A%2A%20Ann%C3%A9e%202026%0A%F0%9F%92%B0%20%2ATotal%20%C3%A0%20r%C3%A9gler%20%3A%2A%20%2A3600%20DH%2A%0A%0A%F0%9F%93%84%20%2AT%C3%A9l%C3%A9charger%20votre%20document%20officiel%20%28PDF%29%20%3A%2A%0A%F0%9F%91%89%20https%3A//srbl.netlify.app/pdf/appel-A01.pdf%0A%0A%F0%9F%8F%A6%20%2ACoordonn%C3%A9es%20bancaires%20pour%20le%20virement%20%3A%2A%0A%E2%80%A2%20%2AB%C3%A9n%C3%A9ficiaire%20%3A%2A%20SYNDICAT%20RESIDENCE%20BELLES%20LOGES%0A%E2%80%A2%20%2ABanque%20%3A%2A%20BMCE%20/%20BANK%20OF%20AFRICA%0A%E2%80%A2%20%2ARIB%20%3A%2A%20%60011%20780%200000402100011545%2025%60%0A%0A_Motif%20%3A%20A01%20-%20ELMOSTAFA%20EL%20GUESSAB_%0A%0AMerci%20pour%20votre%20pr%C3%A9cieuse%20collaboration.%0A%2ALe%20Bureau%20du%20Syndic%2A", "📲 Envoyer WhatsApp Direct")</f>
+        <v/>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>🏢 *SYNDICAT RÉSIDENCE BELLES LOGES*
+📍 Rue Attabari, Quartier Les Princesses, Casablanca
+Bonjour *ELMOSTAFA EL GUESSAB*,
+Veuillez trouver ci-dessous l'appel de cotisations syndicales pour votre bien (*Appartement N°12* / A01) :
+📅 *Période :* Année 2026
+💰 *Total à régler :* *3600 DH*
+📄 *Télécharger votre document officiel (PDF) :*
+👉 https://srbl.netlify.app/pdf/appel-A01.pdf
+🏦 *Coordonnées bancaires pour le virement :*
+• *Bénéficiaire :* SYNDICAT RESIDENCE BELLES LOGES
+• *Banque :* BMCE / BANK OF AFRICA
+• *RIB :* `011 780 0000402100011545 25`
+_Motif : A01 - ELMOSTAFA EL GUESSAB_
+Merci pour votre précieuse collaboration.
+*Le Bureau du Syndic*</t>
+        </is>
+      </c>
+      <c r="Z22" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/?client=A01", "👤 Espace Client (A01)")</f>
+        <v/>
+      </c>
     </row>
     <row r="23" ht="24.95" customHeight="1">
       <c r="B23" s="138" t="inlineStr">
@@ -4241,6 +4801,37 @@
         <f>'Cotisation 2025'!V23</f>
         <v/>
       </c>
+      <c r="W23" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/pdf/appel-A13.pdf", "📄 Voir PDF (A13)")</f>
+        <v/>
+      </c>
+      <c r="X23" s="268">
+        <f>HYPERLINK("https://wa.me/06612148520664908843?text=%F0%9F%8F%A2%20%2ASYNDICAT%20R%C3%89SIDENCE%20BELLES%20LOGES%2A%0A%F0%9F%93%8D%20Rue%20Attabari%2C%20Quartier%20Les%20Princesses%2C%20Casablanca%0A%0ABonjour%20%2ADOUKKALI%20BOUALAM%20ZINEB%20/%20ABDELHADI%20NADIFI%2A%2C%0A%0AVeuillez%20trouver%20ci-dessous%20l%27appel%20de%20cotisations%20syndicales%20pour%20votre%20bien%20%28%2AAppartement%20N%C2%B013%2A%20/%20A13%29%20%3A%0A%0A%F0%9F%93%85%20%2AP%C3%A9riode%20%3A%2A%20Ann%C3%A9e%202026%0A%F0%9F%92%B0%20%2ATotal%20%C3%A0%20r%C3%A9gler%20%3A%2A%20%2A3600%20DH%2A%0A%0A%F0%9F%93%84%20%2AT%C3%A9l%C3%A9charger%20votre%20document%20officiel%20%28PDF%29%20%3A%2A%0A%F0%9F%91%89%20https%3A//srbl.netlify.app/pdf/appel-A13.pdf%0A%0A%F0%9F%8F%A6%20%2ACoordonn%C3%A9es%20bancaires%20pour%20le%20virement%20%3A%2A%0A%E2%80%A2%20%2AB%C3%A9n%C3%A9ficiaire%20%3A%2A%20SYNDICAT%20RESIDENCE%20BELLES%20LOGES%0A%E2%80%A2%20%2ABanque%20%3A%2A%20BMCE%20/%20BANK%20OF%20AFRICA%0A%E2%80%A2%20%2ARIB%20%3A%2A%20%60011%20780%200000402100011545%2025%60%0A%0A_Motif%20%3A%20A13%20-%20DOUKKALI%20BOUALAM%20ZINEB%20/%20ABDELHADI%20NADIFI_%0A%0AMerci%20pour%20votre%20pr%C3%A9cieuse%20collaboration.%0A%2ALe%20Bureau%20du%20Syndic%2A", "📲 Envoyer WhatsApp Direct")</f>
+        <v/>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>🏢 *SYNDICAT RÉSIDENCE BELLES LOGES*
+📍 Rue Attabari, Quartier Les Princesses, Casablanca
+Bonjour *DOUKKALI BOUALAM ZINEB / ABDELHADI NADIFI*,
+Veuillez trouver ci-dessous l'appel de cotisations syndicales pour votre bien (*Appartement N°13* / A13) :
+📅 *Période :* Année 2026
+💰 *Total à régler :* *3600 DH*
+📄 *Télécharger votre document officiel (PDF) :*
+👉 https://srbl.netlify.app/pdf/appel-A13.pdf
+🏦 *Coordonnées bancaires pour le virement :*
+• *Bénéficiaire :* SYNDICAT RESIDENCE BELLES LOGES
+• *Banque :* BMCE / BANK OF AFRICA
+• *RIB :* `011 780 0000402100011545 25`
+_Motif : A13 - DOUKKALI BOUALAM ZINEB / ABDELHADI NADIFI_
+Merci pour votre précieuse collaboration.
+*Le Bureau du Syndic*</t>
+        </is>
+      </c>
+      <c r="Z23" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/?client=A13", "👤 Espace Client (A13)")</f>
+        <v/>
+      </c>
     </row>
     <row r="24" ht="24.75" customFormat="1" customHeight="1" s="34">
       <c r="B24" s="140" t="inlineStr">
@@ -4314,6 +4905,37 @@
         <f>'Cotisation 2025'!V24</f>
         <v/>
       </c>
+      <c r="W24" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/pdf/appel-A14.pdf", "📄 Voir PDF (A14)")</f>
+        <v/>
+      </c>
+      <c r="X24" s="268">
+        <f>HYPERLINK("https://wa.me/06613111650666422524?text=%F0%9F%8F%A2%20%2ASYNDICAT%20R%C3%89SIDENCE%20BELLES%20LOGES%2A%0A%F0%9F%93%8D%20Rue%20Attabari%2C%20Quartier%20Les%20Princesses%2C%20Casablanca%0A%0ABonjour%20%2AGHALLAB%20HAMID%2A%2C%0A%0AVeuillez%20trouver%20ci-dessous%20l%27appel%20de%20cotisations%20syndicales%20pour%20votre%20bien%20%28%2AAppartement%20N%C2%B014%2A%20/%20A14%29%20%3A%0A%0A%F0%9F%93%85%20%2AP%C3%A9riode%20%3A%2A%20Ann%C3%A9e%202026%0A%F0%9F%92%B0%20%2ATotal%20%C3%A0%20r%C3%A9gler%20%3A%2A%20%2A3600%20DH%2A%0A%0A%F0%9F%93%84%20%2AT%C3%A9l%C3%A9charger%20votre%20document%20officiel%20%28PDF%29%20%3A%2A%0A%F0%9F%91%89%20https%3A//srbl.netlify.app/pdf/appel-A14.pdf%0A%0A%F0%9F%8F%A6%20%2ACoordonn%C3%A9es%20bancaires%20pour%20le%20virement%20%3A%2A%0A%E2%80%A2%20%2AB%C3%A9n%C3%A9ficiaire%20%3A%2A%20SYNDICAT%20RESIDENCE%20BELLES%20LOGES%0A%E2%80%A2%20%2ABanque%20%3A%2A%20BMCE%20/%20BANK%20OF%20AFRICA%0A%E2%80%A2%20%2ARIB%20%3A%2A%20%60011%20780%200000402100011545%2025%60%0A%0A_Motif%20%3A%20A14%20-%20GHALLAB%20HAMID_%0A%0AMerci%20pour%20votre%20pr%C3%A9cieuse%20collaboration.%0A%2ALe%20Bureau%20du%20Syndic%2A", "📲 Envoyer WhatsApp Direct")</f>
+        <v/>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>🏢 *SYNDICAT RÉSIDENCE BELLES LOGES*
+📍 Rue Attabari, Quartier Les Princesses, Casablanca
+Bonjour *GHALLAB HAMID*,
+Veuillez trouver ci-dessous l'appel de cotisations syndicales pour votre bien (*Appartement N°14* / A14) :
+📅 *Période :* Année 2026
+💰 *Total à régler :* *3600 DH*
+📄 *Télécharger votre document officiel (PDF) :*
+👉 https://srbl.netlify.app/pdf/appel-A14.pdf
+🏦 *Coordonnées bancaires pour le virement :*
+• *Bénéficiaire :* SYNDICAT RESIDENCE BELLES LOGES
+• *Banque :* BMCE / BANK OF AFRICA
+• *RIB :* `011 780 0000402100011545 25`
+_Motif : A14 - GHALLAB HAMID_
+Merci pour votre précieuse collaboration.
+*Le Bureau du Syndic*</t>
+        </is>
+      </c>
+      <c r="Z24" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/?client=A14", "👤 Espace Client (A14)")</f>
+        <v/>
+      </c>
     </row>
     <row r="25" ht="24.95" customHeight="1">
       <c r="B25" s="128" t="inlineStr">
@@ -4363,13 +4985,13 @@
         <v>300</v>
       </c>
       <c r="P25" s="55" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="Q25" s="55" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="R25" s="55" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="S25" s="126">
         <f>SUM(G25:R25)</f>
@@ -4387,6 +5009,37 @@
         <f>'Cotisation 2025'!V25</f>
         <v/>
       </c>
+      <c r="W25" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/pdf/appel-A15.pdf", "📄 Voir PDF (A15)")</f>
+        <v/>
+      </c>
+      <c r="X25" s="268">
+        <f>HYPERLINK("https://wa.me/212661317078?text=%F0%9F%8F%A2%20%2ASYNDICAT%20R%C3%89SIDENCE%20BELLES%20LOGES%2A%0A%F0%9F%93%8D%20Rue%20Attabari%2C%20Quartier%20Les%20Princesses%2C%20Casablanca%0A%0ABonjour%20%2ADRISS%20BENNANI%2A%2C%0A%0AVeuillez%20trouver%20ci-dessous%20l%27appel%20de%20cotisations%20syndicales%20pour%20votre%20bien%20%28%2AAppartement%20N%C2%B015%2A%20/%20A15%29%20%3A%0A%0A%F0%9F%93%85%20%2AP%C3%A9riode%20%3A%2A%20Ann%C3%A9e%202026%0A%F0%9F%92%B0%20%2ATotal%20%C3%A0%20r%C3%A9gler%20%3A%2A%20%2A3600%20DH%2A%0A%0A%F0%9F%93%84%20%2AT%C3%A9l%C3%A9charger%20votre%20document%20officiel%20%28PDF%29%20%3A%2A%0A%F0%9F%91%89%20https%3A//srbl.netlify.app/pdf/appel-A15.pdf%0A%0A%F0%9F%8F%A6%20%2ACoordonn%C3%A9es%20bancaires%20pour%20le%20virement%20%3A%2A%0A%E2%80%A2%20%2AB%C3%A9n%C3%A9ficiaire%20%3A%2A%20SYNDICAT%20RESIDENCE%20BELLES%20LOGES%0A%E2%80%A2%20%2ABanque%20%3A%2A%20BMCE%20/%20BANK%20OF%20AFRICA%0A%E2%80%A2%20%2ARIB%20%3A%2A%20%60011%20780%200000402100011545%2025%60%0A%0A_Motif%20%3A%20A15%20-%20DRISS%20BENNANI_%0A%0AMerci%20pour%20votre%20pr%C3%A9cieuse%20collaboration.%0A%2ALe%20Bureau%20du%20Syndic%2A", "📲 Envoyer WhatsApp Direct")</f>
+        <v/>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>🏢 *SYNDICAT RÉSIDENCE BELLES LOGES*
+📍 Rue Attabari, Quartier Les Princesses, Casablanca
+Bonjour *DRISS BENNANI*,
+Veuillez trouver ci-dessous l'appel de cotisations syndicales pour votre bien (*Appartement N°15* / A15) :
+📅 *Période :* Année 2026
+💰 *Total à régler :* *3600 DH*
+📄 *Télécharger votre document officiel (PDF) :*
+👉 https://srbl.netlify.app/pdf/appel-A15.pdf
+🏦 *Coordonnées bancaires pour le virement :*
+• *Bénéficiaire :* SYNDICAT RESIDENCE BELLES LOGES
+• *Banque :* BMCE / BANK OF AFRICA
+• *RIB :* `011 780 0000402100011545 25`
+_Motif : A15 - DRISS BENNANI_
+Merci pour votre précieuse collaboration.
+*Le Bureau du Syndic*</t>
+        </is>
+      </c>
+      <c r="Z25" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/?client=A15", "👤 Espace Client (A15)")</f>
+        <v/>
+      </c>
     </row>
     <row r="26" ht="24.95" customHeight="1">
       <c r="B26" s="137" t="inlineStr">
@@ -4436,13 +5089,13 @@
         <v>300</v>
       </c>
       <c r="P26" s="55" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="Q26" s="55" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="R26" s="55" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="S26" s="126">
         <f>SUM(G26:R26)</f>
@@ -4460,6 +5113,37 @@
         <f>'Cotisation 2025'!V26</f>
         <v/>
       </c>
+      <c r="W26" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/pdf/appel-A16.pdf", "📄 Voir PDF (A16)")</f>
+        <v/>
+      </c>
+      <c r="X26" s="268">
+        <f>HYPERLINK("https://wa.me/212661157305?text=%F0%9F%8F%A2%20%2ASYNDICAT%20R%C3%89SIDENCE%20BELLES%20LOGES%2A%0A%F0%9F%93%8D%20Rue%20Attabari%2C%20Quartier%20Les%20Princesses%2C%20Casablanca%0A%0ABonjour%20%2AGHALLAB%20MOUHSSINE%2A%2C%0A%0AVeuillez%20trouver%20ci-dessous%20l%27appel%20de%20cotisations%20syndicales%20pour%20votre%20bien%20%28%2AAppartement%20N%C2%B016%2A%20/%20A16%29%20%3A%0A%0A%F0%9F%93%85%20%2AP%C3%A9riode%20%3A%2A%20Ann%C3%A9e%202026%0A%F0%9F%92%B0%20%2ATotal%20%C3%A0%20r%C3%A9gler%20%3A%2A%20%2A3600%20DH%2A%0A%0A%F0%9F%93%84%20%2AT%C3%A9l%C3%A9charger%20votre%20document%20officiel%20%28PDF%29%20%3A%2A%0A%F0%9F%91%89%20https%3A//srbl.netlify.app/pdf/appel-A16.pdf%0A%0A%F0%9F%8F%A6%20%2ACoordonn%C3%A9es%20bancaires%20pour%20le%20virement%20%3A%2A%0A%E2%80%A2%20%2AB%C3%A9n%C3%A9ficiaire%20%3A%2A%20SYNDICAT%20RESIDENCE%20BELLES%20LOGES%0A%E2%80%A2%20%2ABanque%20%3A%2A%20BMCE%20/%20BANK%20OF%20AFRICA%0A%E2%80%A2%20%2ARIB%20%3A%2A%20%60011%20780%200000402100011545%2025%60%0A%0A_Motif%20%3A%20A16%20-%20GHALLAB%20MOUHSSINE_%0A%0AMerci%20pour%20votre%20pr%C3%A9cieuse%20collaboration.%0A%2ALe%20Bureau%20du%20Syndic%2A", "📲 Envoyer WhatsApp Direct")</f>
+        <v/>
+      </c>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>🏢 *SYNDICAT RÉSIDENCE BELLES LOGES*
+📍 Rue Attabari, Quartier Les Princesses, Casablanca
+Bonjour *GHALLAB MOUHSSINE*,
+Veuillez trouver ci-dessous l'appel de cotisations syndicales pour votre bien (*Appartement N°16* / A16) :
+📅 *Période :* Année 2026
+💰 *Total à régler :* *3600 DH*
+📄 *Télécharger votre document officiel (PDF) :*
+👉 https://srbl.netlify.app/pdf/appel-A16.pdf
+🏦 *Coordonnées bancaires pour le virement :*
+• *Bénéficiaire :* SYNDICAT RESIDENCE BELLES LOGES
+• *Banque :* BMCE / BANK OF AFRICA
+• *RIB :* `011 780 0000402100011545 25`
+_Motif : A16 - GHALLAB MOUHSSINE_
+Merci pour votre précieuse collaboration.
+*Le Bureau du Syndic*</t>
+        </is>
+      </c>
+      <c r="Z26" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/?client=A16", "👤 Espace Client (A16)")</f>
+        <v/>
+      </c>
       <c r="AA26" s="231">
         <f>U40+2640</f>
         <v/>
@@ -4537,6 +5221,37 @@
         <f>'Cotisation 2025'!V27</f>
         <v/>
       </c>
+      <c r="W27" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/pdf/appel-A17.pdf", "📄 Voir PDF (A17)")</f>
+        <v/>
+      </c>
+      <c r="X27" s="268">
+        <f>HYPERLINK("https://wa.me/06613111650666422524?text=%F0%9F%8F%A2%20%2ASYNDICAT%20R%C3%89SIDENCE%20BELLES%20LOGES%2A%0A%F0%9F%93%8D%20Rue%20Attabari%2C%20Quartier%20Les%20Princesses%2C%20Casablanca%0A%0ABonjour%20%2AGHALLAB%20HAMID%2A%2C%0A%0AVeuillez%20trouver%20ci-dessous%20l%27appel%20de%20cotisations%20syndicales%20pour%20votre%20bien%20%28%2AAppartement%20N%C2%B017%2A%20/%20A17%29%20%3A%0A%0A%F0%9F%93%85%20%2AP%C3%A9riode%20%3A%2A%20Ann%C3%A9e%202026%0A%F0%9F%92%B0%20%2ATotal%20%C3%A0%20r%C3%A9gler%20%3A%2A%20%2A3600%20DH%2A%0A%0A%F0%9F%93%84%20%2AT%C3%A9l%C3%A9charger%20votre%20document%20officiel%20%28PDF%29%20%3A%2A%0A%F0%9F%91%89%20https%3A//srbl.netlify.app/pdf/appel-A17.pdf%0A%0A%F0%9F%8F%A6%20%2ACoordonn%C3%A9es%20bancaires%20pour%20le%20virement%20%3A%2A%0A%E2%80%A2%20%2AB%C3%A9n%C3%A9ficiaire%20%3A%2A%20SYNDICAT%20RESIDENCE%20BELLES%20LOGES%0A%E2%80%A2%20%2ABanque%20%3A%2A%20BMCE%20/%20BANK%20OF%20AFRICA%0A%E2%80%A2%20%2ARIB%20%3A%2A%20%60011%20780%200000402100011545%2025%60%0A%0A_Motif%20%3A%20A17%20-%20GHALLAB%20HAMID_%0A%0AMerci%20pour%20votre%20pr%C3%A9cieuse%20collaboration.%0A%2ALe%20Bureau%20du%20Syndic%2A", "📲 Envoyer WhatsApp Direct")</f>
+        <v/>
+      </c>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>🏢 *SYNDICAT RÉSIDENCE BELLES LOGES*
+📍 Rue Attabari, Quartier Les Princesses, Casablanca
+Bonjour *GHALLAB HAMID*,
+Veuillez trouver ci-dessous l'appel de cotisations syndicales pour votre bien (*Appartement N°17* / A17) :
+📅 *Période :* Année 2026
+💰 *Total à régler :* *3600 DH*
+📄 *Télécharger votre document officiel (PDF) :*
+👉 https://srbl.netlify.app/pdf/appel-A17.pdf
+🏦 *Coordonnées bancaires pour le virement :*
+• *Bénéficiaire :* SYNDICAT RESIDENCE BELLES LOGES
+• *Banque :* BMCE / BANK OF AFRICA
+• *RIB :* `011 780 0000402100011545 25`
+_Motif : A17 - GHALLAB HAMID_
+Merci pour votre précieuse collaboration.
+*Le Bureau du Syndic*</t>
+        </is>
+      </c>
+      <c r="Z27" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/?client=A17", "👤 Espace Client (A17)")</f>
+        <v/>
+      </c>
     </row>
     <row r="28" ht="24.95" customHeight="1">
       <c r="B28" s="144" t="inlineStr">
@@ -4610,6 +5325,37 @@
         <f>'Cotisation 2025'!V28</f>
         <v/>
       </c>
+      <c r="W28" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/pdf/appel-A18.pdf", "📄 Voir PDF (A18)")</f>
+        <v/>
+      </c>
+      <c r="X28" s="268">
+        <f>HYPERLINK("https://wa.me/212661324710?text=%F0%9F%8F%A2%20%2ASYNDICAT%20R%C3%89SIDENCE%20BELLES%20LOGES%2A%0A%F0%9F%93%8D%20Rue%20Attabari%2C%20Quartier%20Les%20Princesses%2C%20Casablanca%0A%0ABonjour%20%2AMME%20BEN%20BRAHIM%20ANDALOUSSI%20FATTOUMA%2A%2C%0A%0AVeuillez%20trouver%20ci-dessous%20l%27appel%20de%20cotisations%20syndicales%20pour%20votre%20bien%20%28%2AAppartement%20N%C2%B018%2A%20/%20A18%29%20%3A%0A%0A%F0%9F%93%85%20%2AP%C3%A9riode%20%3A%2A%20Ann%C3%A9e%202026%0A%F0%9F%92%B0%20%2ATotal%20%C3%A0%20r%C3%A9gler%20%3A%2A%20%2A3600%20DH%2A%0A%0A%F0%9F%93%84%20%2AT%C3%A9l%C3%A9charger%20votre%20document%20officiel%20%28PDF%29%20%3A%2A%0A%F0%9F%91%89%20https%3A//srbl.netlify.app/pdf/appel-A18.pdf%0A%0A%F0%9F%8F%A6%20%2ACoordonn%C3%A9es%20bancaires%20pour%20le%20virement%20%3A%2A%0A%E2%80%A2%20%2AB%C3%A9n%C3%A9ficiaire%20%3A%2A%20SYNDICAT%20RESIDENCE%20BELLES%20LOGES%0A%E2%80%A2%20%2ABanque%20%3A%2A%20BMCE%20/%20BANK%20OF%20AFRICA%0A%E2%80%A2%20%2ARIB%20%3A%2A%20%60011%20780%200000402100011545%2025%60%0A%0A_Motif%20%3A%20A18%20-%20MME%20BEN%20BRAHIM%20ANDALOUSSI%20FATTOUMA_%0A%0AMerci%20pour%20votre%20pr%C3%A9cieuse%20collaboration.%0A%2ALe%20Bureau%20du%20Syndic%2A", "📲 Envoyer WhatsApp Direct")</f>
+        <v/>
+      </c>
+      <c r="Y28" t="inlineStr">
+        <is>
+          <t>🏢 *SYNDICAT RÉSIDENCE BELLES LOGES*
+📍 Rue Attabari, Quartier Les Princesses, Casablanca
+Bonjour *MME BEN BRAHIM ANDALOUSSI FATTOUMA*,
+Veuillez trouver ci-dessous l'appel de cotisations syndicales pour votre bien (*Appartement N°18* / A18) :
+📅 *Période :* Année 2026
+💰 *Total à régler :* *3600 DH*
+📄 *Télécharger votre document officiel (PDF) :*
+👉 https://srbl.netlify.app/pdf/appel-A18.pdf
+🏦 *Coordonnées bancaires pour le virement :*
+• *Bénéficiaire :* SYNDICAT RESIDENCE BELLES LOGES
+• *Banque :* BMCE / BANK OF AFRICA
+• *RIB :* `011 780 0000402100011545 25`
+_Motif : A18 - MME BEN BRAHIM ANDALOUSSI FATTOUMA_
+Merci pour votre précieuse collaboration.
+*Le Bureau du Syndic*</t>
+        </is>
+      </c>
+      <c r="Z28" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/?client=A18", "👤 Espace Client (A18)")</f>
+        <v/>
+      </c>
     </row>
     <row r="29" ht="24.95" customHeight="1">
       <c r="B29" s="137" t="inlineStr">
@@ -4661,13 +5407,13 @@
         <v>300</v>
       </c>
       <c r="P29" s="55" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="Q29" s="55" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="R29" s="55" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="S29" s="126">
         <f>SUM(G29:R29)</f>
@@ -4685,6 +5431,37 @@
         <f>'Cotisation 2025'!V29</f>
         <v/>
       </c>
+      <c r="W29" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/pdf/appel-A19.pdf", "📄 Voir PDF (A19)")</f>
+        <v/>
+      </c>
+      <c r="X29" s="268">
+        <f>HYPERLINK("https://wa.me/212661157305?text=%F0%9F%8F%A2%20%2ASYNDICAT%20R%C3%89SIDENCE%20BELLES%20LOGES%2A%0A%F0%9F%93%8D%20Rue%20Attabari%2C%20Quartier%20Les%20Princesses%2C%20Casablanca%0A%0ABonjour%20%2AGHALLAB%20MOUHSSINE%2A%2C%0A%0AVeuillez%20trouver%20ci-dessous%20l%27appel%20de%20cotisations%20syndicales%20pour%20votre%20bien%20%28%2AAppartement%20N%C2%B019%2A%20/%20A19%29%20%3A%0A%0A%F0%9F%93%85%20%2AP%C3%A9riode%20%3A%2A%20Ann%C3%A9e%202026%0A%F0%9F%92%B0%20%2ATotal%20%C3%A0%20r%C3%A9gler%20%3A%2A%20%2A3600%20DH%2A%0A%0A%F0%9F%93%84%20%2AT%C3%A9l%C3%A9charger%20votre%20document%20officiel%20%28PDF%29%20%3A%2A%0A%F0%9F%91%89%20https%3A//srbl.netlify.app/pdf/appel-A19.pdf%0A%0A%F0%9F%8F%A6%20%2ACoordonn%C3%A9es%20bancaires%20pour%20le%20virement%20%3A%2A%0A%E2%80%A2%20%2AB%C3%A9n%C3%A9ficiaire%20%3A%2A%20SYNDICAT%20RESIDENCE%20BELLES%20LOGES%0A%E2%80%A2%20%2ABanque%20%3A%2A%20BMCE%20/%20BANK%20OF%20AFRICA%0A%E2%80%A2%20%2ARIB%20%3A%2A%20%60011%20780%200000402100011545%2025%60%0A%0A_Motif%20%3A%20A19%20-%20GHALLAB%20MOUHSSINE_%0A%0AMerci%20pour%20votre%20pr%C3%A9cieuse%20collaboration.%0A%2ALe%20Bureau%20du%20Syndic%2A", "📲 Envoyer WhatsApp Direct")</f>
+        <v/>
+      </c>
+      <c r="Y29" t="inlineStr">
+        <is>
+          <t>🏢 *SYNDICAT RÉSIDENCE BELLES LOGES*
+📍 Rue Attabari, Quartier Les Princesses, Casablanca
+Bonjour *GHALLAB MOUHSSINE*,
+Veuillez trouver ci-dessous l'appel de cotisations syndicales pour votre bien (*Appartement N°19* / A19) :
+📅 *Période :* Année 2026
+💰 *Total à régler :* *3600 DH*
+📄 *Télécharger votre document officiel (PDF) :*
+👉 https://srbl.netlify.app/pdf/appel-A19.pdf
+🏦 *Coordonnées bancaires pour le virement :*
+• *Bénéficiaire :* SYNDICAT RESIDENCE BELLES LOGES
+• *Banque :* BMCE / BANK OF AFRICA
+• *RIB :* `011 780 0000402100011545 25`
+_Motif : A19 - GHALLAB MOUHSSINE_
+Merci pour votre précieuse collaboration.
+*Le Bureau du Syndic*</t>
+        </is>
+      </c>
+      <c r="Z29" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/?client=A19", "👤 Espace Client (A19)")</f>
+        <v/>
+      </c>
     </row>
     <row r="30" ht="24.95" customHeight="1">
       <c r="B30" s="137" t="inlineStr">
@@ -4758,6 +5535,37 @@
         <f>'Cotisation 2025'!V30</f>
         <v/>
       </c>
+      <c r="W30" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/pdf/appel-A02.pdf", "📄 Voir PDF (A02)")</f>
+        <v/>
+      </c>
+      <c r="X30" s="268">
+        <f>HYPERLINK("https://wa.me/212661157305?text=%F0%9F%8F%A2%20%2ASYNDICAT%20R%C3%89SIDENCE%20BELLES%20LOGES%2A%0A%F0%9F%93%8D%20Rue%20Attabari%2C%20Quartier%20Les%20Princesses%2C%20Casablanca%0A%0ABonjour%20%2AGHALLAB%20MOUHSSINE%2A%2C%0A%0AVeuillez%20trouver%20ci-dessous%20l%27appel%20de%20cotisations%20syndicales%20pour%20votre%20bien%20%28%2AAppartement%20N%C2%B020%2A%20/%20A02%29%20%3A%0A%0A%F0%9F%93%85%20%2AP%C3%A9riode%20%3A%2A%20Ann%C3%A9e%202026%0A%F0%9F%92%B0%20%2ATotal%20%C3%A0%20r%C3%A9gler%20%3A%2A%20%2A3600%20DH%2A%0A%0A%F0%9F%93%84%20%2AT%C3%A9l%C3%A9charger%20votre%20document%20officiel%20%28PDF%29%20%3A%2A%0A%F0%9F%91%89%20https%3A//srbl.netlify.app/pdf/appel-A02.pdf%0A%0A%F0%9F%8F%A6%20%2ACoordonn%C3%A9es%20bancaires%20pour%20le%20virement%20%3A%2A%0A%E2%80%A2%20%2AB%C3%A9n%C3%A9ficiaire%20%3A%2A%20SYNDICAT%20RESIDENCE%20BELLES%20LOGES%0A%E2%80%A2%20%2ABanque%20%3A%2A%20BMCE%20/%20BANK%20OF%20AFRICA%0A%E2%80%A2%20%2ARIB%20%3A%2A%20%60011%20780%200000402100011545%2025%60%0A%0A_Motif%20%3A%20A02%20-%20GHALLAB%20MOUHSSINE_%0A%0AMerci%20pour%20votre%20pr%C3%A9cieuse%20collaboration.%0A%2ALe%20Bureau%20du%20Syndic%2A", "📲 Envoyer WhatsApp Direct")</f>
+        <v/>
+      </c>
+      <c r="Y30" t="inlineStr">
+        <is>
+          <t>🏢 *SYNDICAT RÉSIDENCE BELLES LOGES*
+📍 Rue Attabari, Quartier Les Princesses, Casablanca
+Bonjour *GHALLAB MOUHSSINE*,
+Veuillez trouver ci-dessous l'appel de cotisations syndicales pour votre bien (*Appartement N°20* / A02) :
+📅 *Période :* Année 2026
+💰 *Total à régler :* *3600 DH*
+📄 *Télécharger votre document officiel (PDF) :*
+👉 https://srbl.netlify.app/pdf/appel-A02.pdf
+🏦 *Coordonnées bancaires pour le virement :*
+• *Bénéficiaire :* SYNDICAT RESIDENCE BELLES LOGES
+• *Banque :* BMCE / BANK OF AFRICA
+• *RIB :* `011 780 0000402100011545 25`
+_Motif : A02 - GHALLAB MOUHSSINE_
+Merci pour votre précieuse collaboration.
+*Le Bureau du Syndic*</t>
+        </is>
+      </c>
+      <c r="Z30" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/?client=A02", "👤 Espace Client (A02)")</f>
+        <v/>
+      </c>
     </row>
     <row r="31" ht="24.95" customHeight="1">
       <c r="B31" s="145" t="inlineStr">
@@ -4831,6 +5639,37 @@
         <f>'Cotisation 2025'!V31</f>
         <v/>
       </c>
+      <c r="W31" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/pdf/appel-A02.pdf", "📄 Voir PDF (A02)")</f>
+        <v/>
+      </c>
+      <c r="X31" s="268">
+        <f>HYPERLINK("https://wa.me/212661324710?text=%F0%9F%8F%A2%20%2ASYNDICAT%20R%C3%89SIDENCE%20BELLES%20LOGES%2A%0A%F0%9F%93%8D%20Rue%20Attabari%2C%20Quartier%20Les%20Princesses%2C%20Casablanca%0A%0ABonjour%20%2AMME%20BEN%20BRAHIM%20ANDALOUSSI%20FATTOUMA%2A%2C%0A%0AVeuillez%20trouver%20ci-dessous%20l%27appel%20de%20cotisations%20syndicales%20pour%20votre%20bien%20%28%2AAppartement%20N%C2%B021%2A%20/%20A02%29%20%3A%0A%0A%F0%9F%93%85%20%2AP%C3%A9riode%20%3A%2A%20Ann%C3%A9e%202026%0A%F0%9F%92%B0%20%2ATotal%20%C3%A0%20r%C3%A9gler%20%3A%2A%20%2A3600%20DH%2A%0A%0A%F0%9F%93%84%20%2AT%C3%A9l%C3%A9charger%20votre%20document%20officiel%20%28PDF%29%20%3A%2A%0A%F0%9F%91%89%20https%3A//srbl.netlify.app/pdf/appel-A02.pdf%0A%0A%F0%9F%8F%A6%20%2ACoordonn%C3%A9es%20bancaires%20pour%20le%20virement%20%3A%2A%0A%E2%80%A2%20%2AB%C3%A9n%C3%A9ficiaire%20%3A%2A%20SYNDICAT%20RESIDENCE%20BELLES%20LOGES%0A%E2%80%A2%20%2ABanque%20%3A%2A%20BMCE%20/%20BANK%20OF%20AFRICA%0A%E2%80%A2%20%2ARIB%20%3A%2A%20%60011%20780%200000402100011545%2025%60%0A%0A_Motif%20%3A%20A02%20-%20MME%20BEN%20BRAHIM%20ANDALOUSSI%20FATTOUMA_%0A%0AMerci%20pour%20votre%20pr%C3%A9cieuse%20collaboration.%0A%2ALe%20Bureau%20du%20Syndic%2A", "📲 Envoyer WhatsApp Direct")</f>
+        <v/>
+      </c>
+      <c r="Y31" t="inlineStr">
+        <is>
+          <t>🏢 *SYNDICAT RÉSIDENCE BELLES LOGES*
+📍 Rue Attabari, Quartier Les Princesses, Casablanca
+Bonjour *MME BEN BRAHIM ANDALOUSSI FATTOUMA*,
+Veuillez trouver ci-dessous l'appel de cotisations syndicales pour votre bien (*Appartement N°21* / A02) :
+📅 *Période :* Année 2026
+💰 *Total à régler :* *3600 DH*
+📄 *Télécharger votre document officiel (PDF) :*
+👉 https://srbl.netlify.app/pdf/appel-A02.pdf
+🏦 *Coordonnées bancaires pour le virement :*
+• *Bénéficiaire :* SYNDICAT RESIDENCE BELLES LOGES
+• *Banque :* BMCE / BANK OF AFRICA
+• *RIB :* `011 780 0000402100011545 25`
+_Motif : A02 - MME BEN BRAHIM ANDALOUSSI FATTOUMA_
+Merci pour votre précieuse collaboration.
+*Le Bureau du Syndic*</t>
+        </is>
+      </c>
+      <c r="Z31" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/?client=A02", "👤 Espace Client (A02)")</f>
+        <v/>
+      </c>
     </row>
     <row r="32" ht="24.95" customHeight="1">
       <c r="B32" s="133" t="inlineStr">
@@ -4904,6 +5743,37 @@
         <f>'Cotisation 2025'!V32</f>
         <v/>
       </c>
+      <c r="W32" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/pdf/appel-A02.pdf", "📄 Voir PDF (A02)")</f>
+        <v/>
+      </c>
+      <c r="X32" s="268">
+        <f>HYPERLINK("https://wa.me/212661411823?text=%F0%9F%8F%A2%20%2ASYNDICAT%20R%C3%89SIDENCE%20BELLES%20LOGES%2A%0A%F0%9F%93%8D%20Rue%20Attabari%2C%20Quartier%20Les%20Princesses%2C%20Casablanca%0A%0ABonjour%20%2AGHALLAB%20HAKIM%2A%2C%0A%0AVeuillez%20trouver%20ci-dessous%20l%27appel%20de%20cotisations%20syndicales%20pour%20votre%20bien%20%28%2AAppartement%20N%C2%B022%2A%20/%20A02%29%20%3A%0A%0A%F0%9F%93%85%20%2AP%C3%A9riode%20%3A%2A%20Ann%C3%A9e%202026%0A%F0%9F%92%B0%20%2ATotal%20%C3%A0%20r%C3%A9gler%20%3A%2A%20%2A3600%20DH%2A%0A%0A%F0%9F%93%84%20%2AT%C3%A9l%C3%A9charger%20votre%20document%20officiel%20%28PDF%29%20%3A%2A%0A%F0%9F%91%89%20https%3A//srbl.netlify.app/pdf/appel-A02.pdf%0A%0A%F0%9F%8F%A6%20%2ACoordonn%C3%A9es%20bancaires%20pour%20le%20virement%20%3A%2A%0A%E2%80%A2%20%2AB%C3%A9n%C3%A9ficiaire%20%3A%2A%20SYNDICAT%20RESIDENCE%20BELLES%20LOGES%0A%E2%80%A2%20%2ABanque%20%3A%2A%20BMCE%20/%20BANK%20OF%20AFRICA%0A%E2%80%A2%20%2ARIB%20%3A%2A%20%60011%20780%200000402100011545%2025%60%0A%0A_Motif%20%3A%20A02%20-%20GHALLAB%20HAKIM_%0A%0AMerci%20pour%20votre%20pr%C3%A9cieuse%20collaboration.%0A%2ALe%20Bureau%20du%20Syndic%2A", "📲 Envoyer WhatsApp Direct")</f>
+        <v/>
+      </c>
+      <c r="Y32" t="inlineStr">
+        <is>
+          <t>🏢 *SYNDICAT RÉSIDENCE BELLES LOGES*
+📍 Rue Attabari, Quartier Les Princesses, Casablanca
+Bonjour *GHALLAB HAKIM*,
+Veuillez trouver ci-dessous l'appel de cotisations syndicales pour votre bien (*Appartement N°22* / A02) :
+📅 *Période :* Année 2026
+💰 *Total à régler :* *3600 DH*
+📄 *Télécharger votre document officiel (PDF) :*
+👉 https://srbl.netlify.app/pdf/appel-A02.pdf
+🏦 *Coordonnées bancaires pour le virement :*
+• *Bénéficiaire :* SYNDICAT RESIDENCE BELLES LOGES
+• *Banque :* BMCE / BANK OF AFRICA
+• *RIB :* `011 780 0000402100011545 25`
+_Motif : A02 - GHALLAB HAKIM_
+Merci pour votre précieuse collaboration.
+*Le Bureau du Syndic*</t>
+        </is>
+      </c>
+      <c r="Z32" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/?client=A02", "👤 Espace Client (A02)")</f>
+        <v/>
+      </c>
     </row>
     <row r="33" ht="24.95" customHeight="1">
       <c r="B33" s="128" t="inlineStr">
@@ -4977,6 +5847,37 @@
         <f>'Cotisation 2025'!V33</f>
         <v/>
       </c>
+      <c r="W33" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/pdf/appel-A02.pdf", "📄 Voir PDF (A02)")</f>
+        <v/>
+      </c>
+      <c r="X33" s="268">
+        <f>HYPERLINK("https://wa.me/212606557512?text=%F0%9F%8F%A2%20%2ASYNDICAT%20R%C3%89SIDENCE%20BELLES%20LOGES%2A%0A%F0%9F%93%8D%20Rue%20Attabari%2C%20Quartier%20Les%20Princesses%2C%20Casablanca%0A%0ABonjour%20%2AMOULINE%20LARBI%2A%2C%0A%0AVeuillez%20trouver%20ci-dessous%20l%27appel%20de%20cotisations%20syndicales%20pour%20votre%20bien%20%28%2AAppartement%20N%C2%B023%2A%20/%20A02%29%20%3A%0A%0A%F0%9F%93%85%20%2AP%C3%A9riode%20%3A%2A%20Ann%C3%A9e%202026%0A%F0%9F%92%B0%20%2ATotal%20%C3%A0%20r%C3%A9gler%20%3A%2A%20%2A3600%20DH%2A%0A%0A%F0%9F%93%84%20%2AT%C3%A9l%C3%A9charger%20votre%20document%20officiel%20%28PDF%29%20%3A%2A%0A%F0%9F%91%89%20https%3A//srbl.netlify.app/pdf/appel-A02.pdf%0A%0A%F0%9F%8F%A6%20%2ACoordonn%C3%A9es%20bancaires%20pour%20le%20virement%20%3A%2A%0A%E2%80%A2%20%2AB%C3%A9n%C3%A9ficiaire%20%3A%2A%20SYNDICAT%20RESIDENCE%20BELLES%20LOGES%0A%E2%80%A2%20%2ABanque%20%3A%2A%20BMCE%20/%20BANK%20OF%20AFRICA%0A%E2%80%A2%20%2ARIB%20%3A%2A%20%60011%20780%200000402100011545%2025%60%0A%0A_Motif%20%3A%20A02%20-%20MOULINE%20LARBI_%0A%0AMerci%20pour%20votre%20pr%C3%A9cieuse%20collaboration.%0A%2ALe%20Bureau%20du%20Syndic%2A", "📲 Envoyer WhatsApp Direct")</f>
+        <v/>
+      </c>
+      <c r="Y33" t="inlineStr">
+        <is>
+          <t>🏢 *SYNDICAT RÉSIDENCE BELLES LOGES*
+📍 Rue Attabari, Quartier Les Princesses, Casablanca
+Bonjour *MOULINE LARBI*,
+Veuillez trouver ci-dessous l'appel de cotisations syndicales pour votre bien (*Appartement N°23* / A02) :
+📅 *Période :* Année 2026
+💰 *Total à régler :* *3600 DH*
+📄 *Télécharger votre document officiel (PDF) :*
+👉 https://srbl.netlify.app/pdf/appel-A02.pdf
+🏦 *Coordonnées bancaires pour le virement :*
+• *Bénéficiaire :* SYNDICAT RESIDENCE BELLES LOGES
+• *Banque :* BMCE / BANK OF AFRICA
+• *RIB :* `011 780 0000402100011545 25`
+_Motif : A02 - MOULINE LARBI_
+Merci pour votre précieuse collaboration.
+*Le Bureau du Syndic*</t>
+        </is>
+      </c>
+      <c r="Z33" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/?client=A02", "👤 Espace Client (A02)")</f>
+        <v/>
+      </c>
     </row>
     <row r="34" ht="24.95" customHeight="1">
       <c r="B34" s="136" t="inlineStr">
@@ -5050,6 +5951,37 @@
         <f>'Cotisation 2025'!V34</f>
         <v/>
       </c>
+      <c r="W34" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/pdf/appel-A02.pdf", "📄 Voir PDF (A02)")</f>
+        <v/>
+      </c>
+      <c r="X34" s="268">
+        <f>HYPERLINK("https://wa.me/212669281802?text=%F0%9F%8F%A2%20%2ASYNDICAT%20R%C3%89SIDENCE%20BELLES%20LOGES%2A%0A%F0%9F%93%8D%20Rue%20Attabari%2C%20Quartier%20Les%20Princesses%2C%20Casablanca%0A%0ABonjour%20%2ANMJ%20CAPITAL%20/%20BEN%20HADDOUCH%20YOUNES%2A%2C%0A%0AVeuillez%20trouver%20ci-dessous%20l%27appel%20de%20cotisations%20syndicales%20pour%20votre%20bien%20%28%2AAppartement%20N%C2%B024%2A%20/%20A02%29%20%3A%0A%0A%F0%9F%93%85%20%2AP%C3%A9riode%20%3A%2A%20Ann%C3%A9e%202026%0A%F0%9F%92%B0%20%2ATotal%20%C3%A0%20r%C3%A9gler%20%3A%2A%20%2A3600%20DH%2A%0A%0A%F0%9F%93%84%20%2AT%C3%A9l%C3%A9charger%20votre%20document%20officiel%20%28PDF%29%20%3A%2A%0A%F0%9F%91%89%20https%3A//srbl.netlify.app/pdf/appel-A02.pdf%0A%0A%F0%9F%8F%A6%20%2ACoordonn%C3%A9es%20bancaires%20pour%20le%20virement%20%3A%2A%0A%E2%80%A2%20%2AB%C3%A9n%C3%A9ficiaire%20%3A%2A%20SYNDICAT%20RESIDENCE%20BELLES%20LOGES%0A%E2%80%A2%20%2ABanque%20%3A%2A%20BMCE%20/%20BANK%20OF%20AFRICA%0A%E2%80%A2%20%2ARIB%20%3A%2A%20%60011%20780%200000402100011545%2025%60%0A%0A_Motif%20%3A%20A02%20-%20NMJ%20CAPITAL%20/%20BEN%20HADDOUCH%20YOUNES_%0A%0AMerci%20pour%20votre%20pr%C3%A9cieuse%20collaboration.%0A%2ALe%20Bureau%20du%20Syndic%2A", "📲 Envoyer WhatsApp Direct")</f>
+        <v/>
+      </c>
+      <c r="Y34" t="inlineStr">
+        <is>
+          <t>🏢 *SYNDICAT RÉSIDENCE BELLES LOGES*
+📍 Rue Attabari, Quartier Les Princesses, Casablanca
+Bonjour *NMJ CAPITAL / BEN HADDOUCH YOUNES*,
+Veuillez trouver ci-dessous l'appel de cotisations syndicales pour votre bien (*Appartement N°24* / A02) :
+📅 *Période :* Année 2026
+💰 *Total à régler :* *3600 DH*
+📄 *Télécharger votre document officiel (PDF) :*
+👉 https://srbl.netlify.app/pdf/appel-A02.pdf
+🏦 *Coordonnées bancaires pour le virement :*
+• *Bénéficiaire :* SYNDICAT RESIDENCE BELLES LOGES
+• *Banque :* BMCE / BANK OF AFRICA
+• *RIB :* `011 780 0000402100011545 25`
+_Motif : A02 - NMJ CAPITAL / BEN HADDOUCH YOUNES_
+Merci pour votre précieuse collaboration.
+*Le Bureau du Syndic*</t>
+        </is>
+      </c>
+      <c r="Z34" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/?client=A02", "👤 Espace Client (A02)")</f>
+        <v/>
+      </c>
     </row>
     <row r="35" ht="24.95" customHeight="1">
       <c r="B35" s="128" t="inlineStr">
@@ -5125,6 +6057,37 @@
         <f>'Cotisation 2025'!V35</f>
         <v/>
       </c>
+      <c r="W35" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/pdf/appel-A02.pdf", "📄 Voir PDF (A02)")</f>
+        <v/>
+      </c>
+      <c r="X35" s="268">
+        <f>HYPERLINK("https://wa.me/212661090187?text=%F0%9F%8F%A2%20%2ASYNDICAT%20R%C3%89SIDENCE%20BELLES%20LOGES%2A%0A%F0%9F%93%8D%20Rue%20Attabari%2C%20Quartier%20Les%20Princesses%2C%20Casablanca%0A%0ABonjour%20%2AMME%20HAJJI%20SABAH%2A%2C%0A%0AVeuillez%20trouver%20ci-dessous%20l%27appel%20de%20cotisations%20syndicales%20pour%20votre%20bien%20%28%2AAppartement%20N%C2%B025%2A%20/%20A02%29%20%3A%0A%0A%F0%9F%93%85%20%2AP%C3%A9riode%20%3A%2A%20Ann%C3%A9e%202026%0A%F0%9F%92%B0%20%2ATotal%20%C3%A0%20r%C3%A9gler%20%3A%2A%20%2A3600%20DH%2A%0A%0A%F0%9F%93%84%20%2AT%C3%A9l%C3%A9charger%20votre%20document%20officiel%20%28PDF%29%20%3A%2A%0A%F0%9F%91%89%20https%3A//srbl.netlify.app/pdf/appel-A02.pdf%0A%0A%F0%9F%8F%A6%20%2ACoordonn%C3%A9es%20bancaires%20pour%20le%20virement%20%3A%2A%0A%E2%80%A2%20%2AB%C3%A9n%C3%A9ficiaire%20%3A%2A%20SYNDICAT%20RESIDENCE%20BELLES%20LOGES%0A%E2%80%A2%20%2ABanque%20%3A%2A%20BMCE%20/%20BANK%20OF%20AFRICA%0A%E2%80%A2%20%2ARIB%20%3A%2A%20%60011%20780%200000402100011545%2025%60%0A%0A_Motif%20%3A%20A02%20-%20MME%20HAJJI%20SABAH_%0A%0AMerci%20pour%20votre%20pr%C3%A9cieuse%20collaboration.%0A%2ALe%20Bureau%20du%20Syndic%2A", "📲 Envoyer WhatsApp Direct")</f>
+        <v/>
+      </c>
+      <c r="Y35" t="inlineStr">
+        <is>
+          <t>🏢 *SYNDICAT RÉSIDENCE BELLES LOGES*
+📍 Rue Attabari, Quartier Les Princesses, Casablanca
+Bonjour *MME HAJJI SABAH*,
+Veuillez trouver ci-dessous l'appel de cotisations syndicales pour votre bien (*Appartement N°25* / A02) :
+📅 *Période :* Année 2026
+💰 *Total à régler :* *3600 DH*
+📄 *Télécharger votre document officiel (PDF) :*
+👉 https://srbl.netlify.app/pdf/appel-A02.pdf
+🏦 *Coordonnées bancaires pour le virement :*
+• *Bénéficiaire :* SYNDICAT RESIDENCE BELLES LOGES
+• *Banque :* BMCE / BANK OF AFRICA
+• *RIB :* `011 780 0000402100011545 25`
+_Motif : A02 - MME HAJJI SABAH_
+Merci pour votre précieuse collaboration.
+*Le Bureau du Syndic*</t>
+        </is>
+      </c>
+      <c r="Z35" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/?client=A02", "👤 Espace Client (A02)")</f>
+        <v/>
+      </c>
     </row>
     <row r="36" ht="24.75" customHeight="1">
       <c r="B36" s="128" t="inlineStr">
@@ -5198,6 +6161,37 @@
         <f>'Cotisation 2025'!V36</f>
         <v/>
       </c>
+      <c r="W36" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/pdf/appel-A02.pdf", "📄 Voir PDF (A02)")</f>
+        <v/>
+      </c>
+      <c r="X36" s="268">
+        <f>HYPERLINK("https://wa.me/212661201440?text=%F0%9F%8F%A2%20%2ASYNDICAT%20R%C3%89SIDENCE%20BELLES%20LOGES%2A%0A%F0%9F%93%8D%20Rue%20Attabari%2C%20Quartier%20Les%20Princesses%2C%20Casablanca%0A%0ABonjour%20%2AMLLE%20FILALI%20DOUNIA%2A%2C%0A%0AVeuillez%20trouver%20ci-dessous%20l%27appel%20de%20cotisations%20syndicales%20pour%20votre%20bien%20%28%2AAppartement%20N%C2%B026%2A%20/%20A02%29%20%3A%0A%0A%F0%9F%93%85%20%2AP%C3%A9riode%20%3A%2A%20Ann%C3%A9e%202026%0A%F0%9F%92%B0%20%2ATotal%20%C3%A0%20r%C3%A9gler%20%3A%2A%20%2A3600%20DH%2A%0A%0A%F0%9F%93%84%20%2AT%C3%A9l%C3%A9charger%20votre%20document%20officiel%20%28PDF%29%20%3A%2A%0A%F0%9F%91%89%20https%3A//srbl.netlify.app/pdf/appel-A02.pdf%0A%0A%F0%9F%8F%A6%20%2ACoordonn%C3%A9es%20bancaires%20pour%20le%20virement%20%3A%2A%0A%E2%80%A2%20%2AB%C3%A9n%C3%A9ficiaire%20%3A%2A%20SYNDICAT%20RESIDENCE%20BELLES%20LOGES%0A%E2%80%A2%20%2ABanque%20%3A%2A%20BMCE%20/%20BANK%20OF%20AFRICA%0A%E2%80%A2%20%2ARIB%20%3A%2A%20%60011%20780%200000402100011545%2025%60%0A%0A_Motif%20%3A%20A02%20-%20MLLE%20FILALI%20DOUNIA_%0A%0AMerci%20pour%20votre%20pr%C3%A9cieuse%20collaboration.%0A%2ALe%20Bureau%20du%20Syndic%2A", "📲 Envoyer WhatsApp Direct")</f>
+        <v/>
+      </c>
+      <c r="Y36" t="inlineStr">
+        <is>
+          <t>🏢 *SYNDICAT RÉSIDENCE BELLES LOGES*
+📍 Rue Attabari, Quartier Les Princesses, Casablanca
+Bonjour *MLLE FILALI DOUNIA*,
+Veuillez trouver ci-dessous l'appel de cotisations syndicales pour votre bien (*Appartement N°26* / A02) :
+📅 *Période :* Année 2026
+💰 *Total à régler :* *3600 DH*
+📄 *Télécharger votre document officiel (PDF) :*
+👉 https://srbl.netlify.app/pdf/appel-A02.pdf
+🏦 *Coordonnées bancaires pour le virement :*
+• *Bénéficiaire :* SYNDICAT RESIDENCE BELLES LOGES
+• *Banque :* BMCE / BANK OF AFRICA
+• *RIB :* `011 780 0000402100011545 25`
+_Motif : A02 - MLLE FILALI DOUNIA_
+Merci pour votre précieuse collaboration.
+*Le Bureau du Syndic*</t>
+        </is>
+      </c>
+      <c r="Z36" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/?client=A02", "👤 Espace Client (A02)")</f>
+        <v/>
+      </c>
     </row>
     <row r="37" ht="24.95" customHeight="1">
       <c r="B37" s="128" t="inlineStr">
@@ -5271,6 +6265,37 @@
         <f>'Cotisation 2025'!V37</f>
         <v/>
       </c>
+      <c r="W37" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/pdf/appel-A02.pdf", "📄 Voir PDF (A02)")</f>
+        <v/>
+      </c>
+      <c r="X37" s="268">
+        <f>HYPERLINK("https://wa.me/212663381883?text=%F0%9F%8F%A2%20%2ASYNDICAT%20R%C3%89SIDENCE%20BELLES%20LOGES%2A%0A%F0%9F%93%8D%20Rue%20Attabari%2C%20Quartier%20Les%20Princesses%2C%20Casablanca%0A%0ABonjour%20%2AMME%20AAMARA%20HAKIMA/MOUFARREH%20ADIL%2A%2C%0A%0AVeuillez%20trouver%20ci-dessous%20l%27appel%20de%20cotisations%20syndicales%20pour%20votre%20bien%20%28%2AAppartement%20N%C2%B027%2A%20/%20A02%29%20%3A%0A%0A%F0%9F%93%85%20%2AP%C3%A9riode%20%3A%2A%20Ann%C3%A9e%202026%0A%F0%9F%92%B0%20%2ATotal%20%C3%A0%20r%C3%A9gler%20%3A%2A%20%2A3600%20DH%2A%0A%0A%F0%9F%93%84%20%2AT%C3%A9l%C3%A9charger%20votre%20document%20officiel%20%28PDF%29%20%3A%2A%0A%F0%9F%91%89%20https%3A//srbl.netlify.app/pdf/appel-A02.pdf%0A%0A%F0%9F%8F%A6%20%2ACoordonn%C3%A9es%20bancaires%20pour%20le%20virement%20%3A%2A%0A%E2%80%A2%20%2AB%C3%A9n%C3%A9ficiaire%20%3A%2A%20SYNDICAT%20RESIDENCE%20BELLES%20LOGES%0A%E2%80%A2%20%2ABanque%20%3A%2A%20BMCE%20/%20BANK%20OF%20AFRICA%0A%E2%80%A2%20%2ARIB%20%3A%2A%20%60011%20780%200000402100011545%2025%60%0A%0A_Motif%20%3A%20A02%20-%20MME%20AAMARA%20HAKIMA/MOUFARREH%20ADIL_%0A%0AMerci%20pour%20votre%20pr%C3%A9cieuse%20collaboration.%0A%2ALe%20Bureau%20du%20Syndic%2A", "📲 Envoyer WhatsApp Direct")</f>
+        <v/>
+      </c>
+      <c r="Y37" t="inlineStr">
+        <is>
+          <t>🏢 *SYNDICAT RÉSIDENCE BELLES LOGES*
+📍 Rue Attabari, Quartier Les Princesses, Casablanca
+Bonjour *MME AAMARA HAKIMA/MOUFARREH ADIL*,
+Veuillez trouver ci-dessous l'appel de cotisations syndicales pour votre bien (*Appartement N°27* / A02) :
+📅 *Période :* Année 2026
+💰 *Total à régler :* *3600 DH*
+📄 *Télécharger votre document officiel (PDF) :*
+👉 https://srbl.netlify.app/pdf/appel-A02.pdf
+🏦 *Coordonnées bancaires pour le virement :*
+• *Bénéficiaire :* SYNDICAT RESIDENCE BELLES LOGES
+• *Banque :* BMCE / BANK OF AFRICA
+• *RIB :* `011 780 0000402100011545 25`
+_Motif : A02 - MME AAMARA HAKIMA/MOUFARREH ADIL_
+Merci pour votre précieuse collaboration.
+*Le Bureau du Syndic*</t>
+        </is>
+      </c>
+      <c r="Z37" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/?client=A02", "👤 Espace Client (A02)")</f>
+        <v/>
+      </c>
     </row>
     <row r="38" ht="24.75" customHeight="1">
       <c r="B38" s="128" t="inlineStr">
@@ -5344,6 +6369,37 @@
         <f>'Cotisation 2025'!V38</f>
         <v/>
       </c>
+      <c r="W38" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/pdf/appel-A02.pdf", "📄 Voir PDF (A02)")</f>
+        <v/>
+      </c>
+      <c r="X38" s="268">
+        <f>HYPERLINK("https://wa.me/212661478244?text=%F0%9F%8F%A2%20%2ASYNDICAT%20R%C3%89SIDENCE%20BELLES%20LOGES%2A%0A%F0%9F%93%8D%20Rue%20Attabari%2C%20Quartier%20Les%20Princesses%2C%20Casablanca%0A%0ABonjour%20%2AYASSINE%20YATRIBI%2A%2C%0A%0AVeuillez%20trouver%20ci-dessous%20l%27appel%20de%20cotisations%20syndicales%20pour%20votre%20bien%20%28%2AAppartement%20N%C2%B028%2A%20/%20A02%29%20%3A%0A%0A%F0%9F%93%85%20%2AP%C3%A9riode%20%3A%2A%20Ann%C3%A9e%202026%0A%F0%9F%92%B0%20%2ATotal%20%C3%A0%20r%C3%A9gler%20%3A%2A%20%2A3600%20DH%2A%0A%0A%F0%9F%93%84%20%2AT%C3%A9l%C3%A9charger%20votre%20document%20officiel%20%28PDF%29%20%3A%2A%0A%F0%9F%91%89%20https%3A//srbl.netlify.app/pdf/appel-A02.pdf%0A%0A%F0%9F%8F%A6%20%2ACoordonn%C3%A9es%20bancaires%20pour%20le%20virement%20%3A%2A%0A%E2%80%A2%20%2AB%C3%A9n%C3%A9ficiaire%20%3A%2A%20SYNDICAT%20RESIDENCE%20BELLES%20LOGES%0A%E2%80%A2%20%2ABanque%20%3A%2A%20BMCE%20/%20BANK%20OF%20AFRICA%0A%E2%80%A2%20%2ARIB%20%3A%2A%20%60011%20780%200000402100011545%2025%60%0A%0A_Motif%20%3A%20A02%20-%20YASSINE%20YATRIBI_%0A%0AMerci%20pour%20votre%20pr%C3%A9cieuse%20collaboration.%0A%2ALe%20Bureau%20du%20Syndic%2A", "📲 Envoyer WhatsApp Direct")</f>
+        <v/>
+      </c>
+      <c r="Y38" t="inlineStr">
+        <is>
+          <t>🏢 *SYNDICAT RÉSIDENCE BELLES LOGES*
+📍 Rue Attabari, Quartier Les Princesses, Casablanca
+Bonjour *YASSINE YATRIBI*,
+Veuillez trouver ci-dessous l'appel de cotisations syndicales pour votre bien (*Appartement N°28* / A02) :
+📅 *Période :* Année 2026
+💰 *Total à régler :* *3600 DH*
+📄 *Télécharger votre document officiel (PDF) :*
+👉 https://srbl.netlify.app/pdf/appel-A02.pdf
+🏦 *Coordonnées bancaires pour le virement :*
+• *Bénéficiaire :* SYNDICAT RESIDENCE BELLES LOGES
+• *Banque :* BMCE / BANK OF AFRICA
+• *RIB :* `011 780 0000402100011545 25`
+_Motif : A02 - YASSINE YATRIBI_
+Merci pour votre précieuse collaboration.
+*Le Bureau du Syndic*</t>
+        </is>
+      </c>
+      <c r="Z38" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/?client=A02", "👤 Espace Client (A02)")</f>
+        <v/>
+      </c>
     </row>
     <row r="39" ht="24.95" customHeight="1">
       <c r="B39" s="128" t="inlineStr">
@@ -5415,6 +6471,37 @@
       </c>
       <c r="V39" s="127">
         <f>'Cotisation 2025'!V39</f>
+        <v/>
+      </c>
+      <c r="W39" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/pdf/appel-A02.pdf", "📄 Voir PDF (A02)")</f>
+        <v/>
+      </c>
+      <c r="X39" s="268">
+        <f>HYPERLINK("https://wa.me/212661457372?text=%F0%9F%8F%A2%20%2ASYNDICAT%20R%C3%89SIDENCE%20BELLES%20LOGES%2A%0A%F0%9F%93%8D%20Rue%20Attabari%2C%20Quartier%20Les%20Princesses%2C%20Casablanca%0A%0ABonjour%20%2AMAMOUNE%20KETTANI%2A%2C%0A%0AVeuillez%20trouver%20ci-dessous%20l%27appel%20de%20cotisations%20syndicales%20pour%20votre%20bien%20%28%2AAppartement%20N%C2%B029%2A%20/%20A02%29%20%3A%0A%0A%F0%9F%93%85%20%2AP%C3%A9riode%20%3A%2A%20Ann%C3%A9e%202026%0A%F0%9F%92%B0%20%2ATotal%20%C3%A0%20r%C3%A9gler%20%3A%2A%20%2A3600%20DH%2A%0A%0A%F0%9F%93%84%20%2AT%C3%A9l%C3%A9charger%20votre%20document%20officiel%20%28PDF%29%20%3A%2A%0A%F0%9F%91%89%20https%3A//srbl.netlify.app/pdf/appel-A02.pdf%0A%0A%F0%9F%8F%A6%20%2ACoordonn%C3%A9es%20bancaires%20pour%20le%20virement%20%3A%2A%0A%E2%80%A2%20%2AB%C3%A9n%C3%A9ficiaire%20%3A%2A%20SYNDICAT%20RESIDENCE%20BELLES%20LOGES%0A%E2%80%A2%20%2ABanque%20%3A%2A%20BMCE%20/%20BANK%20OF%20AFRICA%0A%E2%80%A2%20%2ARIB%20%3A%2A%20%60011%20780%200000402100011545%2025%60%0A%0A_Motif%20%3A%20A02%20-%20MAMOUNE%20KETTANI_%0A%0AMerci%20pour%20votre%20pr%C3%A9cieuse%20collaboration.%0A%2ALe%20Bureau%20du%20Syndic%2A", "📲 Envoyer WhatsApp Direct")</f>
+        <v/>
+      </c>
+      <c r="Y39" t="inlineStr">
+        <is>
+          <t>🏢 *SYNDICAT RÉSIDENCE BELLES LOGES*
+📍 Rue Attabari, Quartier Les Princesses, Casablanca
+Bonjour *MAMOUNE KETTANI*,
+Veuillez trouver ci-dessous l'appel de cotisations syndicales pour votre bien (*Appartement N°29* / A02) :
+📅 *Période :* Année 2026
+💰 *Total à régler :* *3600 DH*
+📄 *Télécharger votre document officiel (PDF) :*
+👉 https://srbl.netlify.app/pdf/appel-A02.pdf
+🏦 *Coordonnées bancaires pour le virement :*
+• *Bénéficiaire :* SYNDICAT RESIDENCE BELLES LOGES
+• *Banque :* BMCE / BANK OF AFRICA
+• *RIB :* `011 780 0000402100011545 25`
+_Motif : A02 - MAMOUNE KETTANI_
+Merci pour votre précieuse collaboration.
+*Le Bureau du Syndic*</t>
+        </is>
+      </c>
+      <c r="Z39" s="267">
+        <f>HYPERLINK("https://srbl.netlify.app/?client=A02", "👤 Espace Client (A02)")</f>
         <v/>
       </c>
     </row>

</xml_diff>